<commit_message>
added work on calculating and printing to file the synced blink percent for dyads and triads
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,14 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFA9684-43EF-4D7B-ABEB-16DA5D1160CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB40E47-D377-4711-B6D3-9B86D6CBF8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="165" yWindow="240" windowWidth="28635" windowHeight="15240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="BlinkRateMinute" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet2!$D$3</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet2!$D$4:$D$13</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$E$3</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$E$4:$E$13</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$D$3</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet2!$D$4:$D$13</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet2!$E$3</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet2!$E$4:$E$13</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="143">
   <si>
     <t>Group</t>
   </si>
@@ -460,13 +471,19 @@
   </si>
   <si>
     <t>X Variable 1</t>
+  </si>
+  <si>
+    <t>Dyad</t>
+  </si>
+  <si>
+    <t>Triad</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -491,6 +508,12 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -542,18 +565,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -561,8 +580,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -573,26 +601,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="14">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9.8000000000000007"/>
-        <color auto="1"/>
-        <name val="JetBrains Mono"/>
-        <family val="3"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -766,6 +774,26 @@
         <family val="3"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9.8000000000000007"/>
+        <color auto="1"/>
+        <name val="JetBrains Mono"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -994,38 +1022,6 @@
                   <c:y val="-0.11867498065631969"/>
                 </c:manualLayout>
               </c:layout>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr>
-                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                        <a:solidFill>
-                          <a:schemeClr val="tx1">
-                            <a:lumMod val="65000"/>
-                            <a:lumOff val="35000"/>
-                          </a:schemeClr>
-                        </a:solidFill>
-                        <a:latin typeface="+mn-lt"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:defRPr>
-                    </a:pPr>
-                    <a:r>
-                      <a:rPr lang="en-US" baseline="0"/>
-                      <a:t>r=-0.072, p=</a:t>
-                    </a:r>
-                    <a:r>
-                      <a:rPr lang="en-GB" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                        <a:effectLst/>
-                      </a:rPr>
-                      <a:t>.988</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -4488,6 +4484,71 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.1</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.3</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0"/>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{5F5FEFE0-8F79-4C9C-BDD4-A3321F378915}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.0</cx:f>
+              <cx:v>Dyad</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:noFill/>
+          </cx:spPr>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="1" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{3BB713B9-C79C-4E48-A5E2-750F24D24DB1}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.2</cx:f>
+              <cx:v>Triad</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:noFill/>
+          </cx:spPr>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="1" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -4808,6 +4869,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -8932,6 +9033,521 @@
         <a:noFill/>
       </a:ln>
     </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -9239,14 +9855,97 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>471487</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>166687</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C091EC3-4082-B497-BD51-15A1FFB0C187}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4738687" y="200025"/>
+              <a:ext cx="4572000" cy="2752725"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-GB" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AD080257-BFA1-460B-B07A-36A64761A16A}" name="Table1" displayName="Table1" ref="C1:F11" totalsRowShown="0" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AD080257-BFA1-460B-B07A-36A64761A16A}" name="Table1" displayName="Table1" ref="C1:F11" totalsRowShown="0" dataDxfId="13">
   <autoFilter ref="C1:F11" xr:uid="{AD080257-BFA1-460B-B07A-36A64761A16A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{4F27821A-74B4-4054-BD57-59CB04F69638}" name="Group" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{40FF8A35-FADD-40F8-9C7C-8272D131492D}" name="P1" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{57E54AEA-9EE5-4960-BBF2-37C5CACE9F4B}" name="P2" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{9B5C91BC-FC38-40B1-900E-1D679A89BBE9}" name="P1_P2_AVG" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{4F27821A-74B4-4054-BD57-59CB04F69638}" name="Group" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{40FF8A35-FADD-40F8-9C7C-8272D131492D}" name="P1" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{57E54AEA-9EE5-4960-BBF2-37C5CACE9F4B}" name="P2" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{9B5C91BC-FC38-40B1-900E-1D679A89BBE9}" name="P1_P2_AVG" dataDxfId="9">
       <calculatedColumnFormula>AVERAGE(Table1[[#This Row],[P1]]:Table1[[#This Row],[P2]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9255,20 +9954,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1613B083-0BCB-449A-A18A-943282863FFE}" name="Table2" displayName="Table2" ref="I1:P10" totalsRowShown="0" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1613B083-0BCB-449A-A18A-943282863FFE}" name="Table2" displayName="Table2" ref="I1:P10" totalsRowShown="0" dataDxfId="8">
   <autoFilter ref="I1:P10" xr:uid="{1613B083-0BCB-449A-A18A-943282863FFE}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{4B00F100-EEAB-4176-8F7C-64576AF95E9C}" name="Group" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{0C1C6D39-9F0B-4EFB-8FFF-6819FFEE1A73}" name="P1" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{4B646295-E6BA-4208-9890-BF77B7CC4DB0}" name="P2" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{90141FC2-ED7D-4A6B-AFC1-04A51D13EAB7}" name="P3" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{45EA91F4-80A5-4D09-8BA5-58CA8E684F50}" name="avg_P1P2" dataDxfId="4">
+    <tableColumn id="1" xr3:uid="{4B00F100-EEAB-4176-8F7C-64576AF95E9C}" name="Group" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{0C1C6D39-9F0B-4EFB-8FFF-6819FFEE1A73}" name="P1" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{4B646295-E6BA-4208-9890-BF77B7CC4DB0}" name="P2" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{90141FC2-ED7D-4A6B-AFC1-04A51D13EAB7}" name="P3" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{45EA91F4-80A5-4D09-8BA5-58CA8E684F50}" name="avg_P1P2" dataDxfId="3">
       <calculatedColumnFormula>AVERAGE(Table2[[#This Row],[P1]:[P2]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8D95483F-1D1F-4BC0-9A13-DB0617692381}" name="avg_P1P3" dataDxfId="3">
+    <tableColumn id="6" xr3:uid="{8D95483F-1D1F-4BC0-9A13-DB0617692381}" name="avg_P1P3" dataDxfId="2">
       <calculatedColumnFormula>AVERAGE(J2,L2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{CEE85F33-BF2F-4114-920C-22ACF0374CF1}" name="avg_P2P3" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{CEE85F33-BF2F-4114-920C-22ACF0374CF1}" name="avg_P2P3" dataDxfId="1">
       <calculatedColumnFormula>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{2974D60E-6187-4B53-9C0A-D6CCD473C533}" name="avg_P123" dataDxfId="0">
@@ -9543,13 +10242,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="54.6328125" customWidth="1"/>
-    <col min="2" max="2" width="22.81640625" customWidth="1"/>
+    <col min="1" max="1" width="54.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="10.81640625" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -10010,15 +10709,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08CBB891-F584-4F5A-A553-41469C7D6F94}">
-  <dimension ref="C1:AA125"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="C1:AA116"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="57.1796875" customWidth="1"/>
+    <col min="3" max="3" width="57.140625" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="9" max="9" width="58.26953125" customWidth="1"/>
+    <col min="9" max="9" width="58.28515625" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" customWidth="1"/>
-    <col min="15" max="15" width="11.90625" customWidth="1"/>
+    <col min="14" max="15" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:16">
@@ -10063,7 +10761,7 @@
       <c r="C2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="7">
         <v>2.4711409999999998</v>
       </c>
       <c r="E2" s="2">
@@ -10097,7 +10795,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>31.417258499999999</v>
       </c>
-      <c r="P2" s="3">
+      <c r="P2" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>25.371325666666667</v>
       </c>
@@ -10140,7 +10838,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>22.229472000000001</v>
       </c>
-      <c r="P3" s="3">
+      <c r="P3" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>20.852425</v>
       </c>
@@ -10162,7 +10860,7 @@
       <c r="I4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="7">
         <v>2.2134100000000001</v>
       </c>
       <c r="K4" s="2">
@@ -10183,7 +10881,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>17.035349</v>
       </c>
-      <c r="P4" s="3">
+      <c r="P4" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>12.094702666666668</v>
       </c>
@@ -10211,7 +10909,7 @@
       <c r="K5" s="2">
         <v>7.7812380000000001</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="7">
         <v>58.124909000000002</v>
       </c>
       <c r="M5" s="2">
@@ -10226,7 +10924,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>32.953073500000002</v>
       </c>
-      <c r="P5" s="3">
+      <c r="P5" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>30.031203000000001</v>
       </c>
@@ -10269,7 +10967,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>16.420914499999999</v>
       </c>
-      <c r="P6" s="3">
+      <c r="P6" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>15.313345666666665</v>
       </c>
@@ -10312,7 +11010,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>8.344597499999999</v>
       </c>
-      <c r="P7" s="3">
+      <c r="P7" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>8.8733186666666661</v>
       </c>
@@ -10355,7 +11053,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>10.815789499999999</v>
       </c>
-      <c r="P8" s="3">
+      <c r="P8" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>13.473684333333333</v>
       </c>
@@ -10398,7 +11096,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>30.613771999999997</v>
       </c>
-      <c r="P9" s="3">
+      <c r="P9" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>24.944554999999998</v>
       </c>
@@ -10441,7 +11139,7 @@
         <f>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</f>
         <v>14.0127335</v>
       </c>
-      <c r="P10" s="3">
+      <c r="P10" s="2">
         <f>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</f>
         <v>19.701947333333333</v>
       </c>
@@ -10472,137 +11170,90 @@
         <v>-7.203443722093221E-2</v>
       </c>
     </row>
-    <row r="23" spans="11:27" ht="15" thickBot="1"/>
+    <row r="23" spans="11:27" ht="15.75" thickBot="1"/>
     <row r="24" spans="11:27">
-      <c r="Y24" s="6"/>
-      <c r="Z24" s="6"/>
-      <c r="AA24" s="6"/>
-    </row>
-    <row r="25" spans="11:27">
-      <c r="Y25" s="4"/>
-      <c r="Z25" s="4"/>
-      <c r="AA25" s="4"/>
-    </row>
-    <row r="26" spans="11:27">
-      <c r="Y26" s="4"/>
-      <c r="Z26" s="4"/>
-      <c r="AA26" s="4"/>
-    </row>
-    <row r="27" spans="11:27">
-      <c r="Y27" s="4"/>
-      <c r="Z27" s="4"/>
-      <c r="AA27" s="4"/>
-    </row>
-    <row r="28" spans="11:27">
-      <c r="Y28" s="4"/>
-      <c r="Z28" s="4"/>
-      <c r="AA28" s="4"/>
-    </row>
-    <row r="29" spans="11:27">
-      <c r="Y29" s="4"/>
-      <c r="Z29" s="4"/>
-      <c r="AA29" s="4"/>
-    </row>
-    <row r="30" spans="11:27">
-      <c r="Y30" s="4"/>
-      <c r="Z30" s="4"/>
-      <c r="AA30" s="4"/>
-    </row>
-    <row r="31" spans="11:27">
-      <c r="Y31" s="4"/>
-      <c r="Z31" s="4"/>
-      <c r="AA31" s="4"/>
+      <c r="Y24" s="4"/>
+      <c r="Z24" s="4"/>
+      <c r="AA24" s="4"/>
     </row>
     <row r="32" spans="11:27">
-      <c r="K32" s="8" t="s">
+      <c r="K32" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="Y32" s="4"/>
-      <c r="Z32" s="4"/>
-      <c r="AA32" s="4"/>
-    </row>
-    <row r="33" spans="4:27" ht="15" thickBot="1">
-      <c r="K33" s="7" t="s">
+    </row>
+    <row r="33" spans="4:27" ht="15.75" thickBot="1">
+      <c r="K33" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="Y33" s="4"/>
-      <c r="Z33" s="4"/>
-      <c r="AA33" s="4"/>
     </row>
     <row r="34" spans="4:27">
-      <c r="K34" s="6"/>
-      <c r="L34" s="6" t="s">
+      <c r="K34" s="4"/>
+      <c r="L34" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="M34" s="6" t="s">
+      <c r="M34" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="Y34" s="4"/>
-      <c r="Z34" s="4"/>
-      <c r="AA34" s="4"/>
-    </row>
-    <row r="35" spans="4:27" ht="15" thickBot="1">
-      <c r="K35" s="4" t="s">
+    </row>
+    <row r="35" spans="4:27" ht="15.75" thickBot="1">
+      <c r="K35" t="s">
         <v>99</v>
       </c>
-      <c r="L35" s="4">
+      <c r="L35">
         <v>18.961834148148149</v>
       </c>
-      <c r="M35" s="4">
+      <c r="M35">
         <v>28.455410500000006</v>
       </c>
-      <c r="Y35" s="5"/>
-      <c r="Z35" s="5"/>
-      <c r="AA35" s="5"/>
+      <c r="Y35" s="3"/>
+      <c r="Z35" s="3"/>
+      <c r="AA35" s="3"/>
     </row>
     <row r="36" spans="4:27">
-      <c r="K36" s="4" t="s">
+      <c r="K36" t="s">
         <v>100</v>
       </c>
-      <c r="L36" s="4">
+      <c r="L36">
         <v>49.486806798110422</v>
       </c>
-      <c r="M36" s="4">
+      <c r="M36">
         <v>80.447471020117121</v>
       </c>
     </row>
     <row r="37" spans="4:27">
-      <c r="K37" s="4" t="s">
+      <c r="K37" t="s">
         <v>101</v>
       </c>
-      <c r="L37" s="4">
+      <c r="L37">
         <v>9</v>
       </c>
-      <c r="M37" s="4">
+      <c r="M37">
         <v>10</v>
       </c>
     </row>
     <row r="38" spans="4:27">
-      <c r="K38" s="4" t="s">
+      <c r="K38" t="s">
         <v>102</v>
       </c>
-      <c r="L38" s="4">
+      <c r="L38">
         <v>0</v>
       </c>
-      <c r="M38" s="4"/>
     </row>
     <row r="39" spans="4:27">
-      <c r="K39" s="4" t="s">
+      <c r="K39" t="s">
         <v>103</v>
       </c>
-      <c r="L39" s="4">
+      <c r="L39">
         <v>17</v>
       </c>
-      <c r="M39" s="4"/>
     </row>
     <row r="40" spans="4:27">
-      <c r="K40" s="4" t="s">
+      <c r="K40" t="s">
         <v>104</v>
       </c>
-      <c r="L40" s="4">
+      <c r="L40">
         <v>-2.5796922549107779</v>
       </c>
-      <c r="M40" s="4"/>
       <c r="Q40" t="s">
         <v>112</v>
       </c>
@@ -10611,84 +11262,81 @@
       </c>
     </row>
     <row r="41" spans="4:27">
-      <c r="K41" s="4" t="s">
+      <c r="K41" t="s">
         <v>105</v>
       </c>
-      <c r="L41" s="4">
+      <c r="L41">
         <v>9.740265652592138E-3</v>
       </c>
-      <c r="M41" s="4"/>
       <c r="Q41">
         <v>13.27946</v>
       </c>
       <c r="R41">
         <v>2.4711409999999998</v>
       </c>
-      <c r="U41" s="8" t="s">
+      <c r="U41" s="6" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="4:27" ht="15" thickBot="1">
-      <c r="K42" s="4" t="s">
+    <row r="42" spans="4:27" ht="15.75" thickBot="1">
+      <c r="K42" t="s">
         <v>106</v>
       </c>
-      <c r="L42" s="4">
+      <c r="L42">
         <v>1.7396067260750732</v>
       </c>
-      <c r="M42" s="4"/>
       <c r="Q42">
         <v>18.098331000000002</v>
       </c>
       <c r="R42">
         <v>32.792991000000001</v>
       </c>
-      <c r="U42" s="7" t="s">
+      <c r="U42" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="43" spans="4:27">
-      <c r="K43" s="4" t="s">
+      <c r="K43" t="s">
         <v>107</v>
       </c>
-      <c r="L43" s="4">
+      <c r="L43">
         <v>1.9480531305184276E-2</v>
       </c>
-      <c r="M43" s="4"/>
       <c r="Q43">
         <v>2.2134100000000001</v>
       </c>
       <c r="R43">
         <v>32.033904</v>
       </c>
-      <c r="U43" s="6"/>
-      <c r="V43" s="6" t="s">
+      <c r="U43" s="4"/>
+      <c r="V43" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="W43" s="6" t="s">
+      <c r="W43" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="4:27" ht="15" thickBot="1">
-      <c r="K44" s="5" t="s">
+    <row r="44" spans="4:27" ht="15.75" thickBot="1">
+      <c r="K44" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="L44" s="5">
+      <c r="L44" s="3">
         <v>2.109815577833317</v>
       </c>
-      <c r="M44" s="5"/>
+      <c r="M44" s="3"/>
       <c r="Q44">
         <v>24.187462</v>
       </c>
       <c r="R44">
         <v>38.272494999999999</v>
       </c>
-      <c r="U44" s="4" t="s">
+      <c r="U44" t="s">
         <v>99</v>
       </c>
-      <c r="V44" s="4">
+      <c r="V44">
         <v>18.961834148148146</v>
       </c>
-      <c r="W44" s="4">
+      <c r="W44">
         <v>28.455410499999999</v>
       </c>
     </row>
@@ -10699,13 +11347,13 @@
       <c r="R45">
         <v>17.652170000000002</v>
       </c>
-      <c r="U45" s="4" t="s">
+      <c r="U45" t="s">
         <v>100</v>
       </c>
-      <c r="V45" s="4">
+      <c r="V45">
         <v>144.02790603704489</v>
       </c>
-      <c r="W45" s="4">
+      <c r="W45">
         <v>171.30275626533091</v>
       </c>
     </row>
@@ -10716,18 +11364,18 @@
       <c r="R46">
         <v>13.541086</v>
       </c>
-      <c r="U46" s="4" t="s">
+      <c r="U46" t="s">
         <v>101</v>
       </c>
-      <c r="V46" s="4">
+      <c r="V46">
         <v>27</v>
       </c>
-      <c r="W46" s="4">
+      <c r="W46">
         <v>20</v>
       </c>
     </row>
     <row r="47" spans="4:27">
-      <c r="K47" s="8" t="s">
+      <c r="K47" s="6" t="s">
         <v>110</v>
       </c>
       <c r="Q47">
@@ -10736,22 +11384,21 @@
       <c r="R47">
         <v>22.615593000000001</v>
       </c>
-      <c r="U47" s="4" t="s">
+      <c r="U47" t="s">
         <v>111</v>
       </c>
-      <c r="V47" s="4">
+      <c r="V47">
         <v>155.54395391121008</v>
       </c>
-      <c r="W47" s="4"/>
-    </row>
-    <row r="48" spans="4:27" ht="15" thickBot="1">
+    </row>
+    <row r="48" spans="4:27" ht="15.75" thickBot="1">
       <c r="D48">
         <v>2.4711409999999998</v>
       </c>
       <c r="E48">
         <v>30.938687999999999</v>
       </c>
-      <c r="K48" s="7" t="s">
+      <c r="K48" s="5" t="s">
         <v>115</v>
       </c>
       <c r="Q48">
@@ -10760,13 +11407,12 @@
       <c r="R48">
         <v>60.294035000000001</v>
       </c>
-      <c r="U48" s="4" t="s">
+      <c r="U48" t="s">
         <v>102</v>
       </c>
-      <c r="V48" s="4">
+      <c r="V48">
         <v>0</v>
       </c>
-      <c r="W48" s="4"/>
     </row>
     <row r="49" spans="4:23">
       <c r="D49">
@@ -10775,11 +11421,11 @@
       <c r="E49">
         <v>31.456980000000001</v>
       </c>
-      <c r="K49" s="6"/>
-      <c r="L49" s="6" t="s">
+      <c r="K49" s="4"/>
+      <c r="L49" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="M49" s="6" t="s">
+      <c r="M49" s="4" t="s">
         <v>98</v>
       </c>
       <c r="Q49">
@@ -10788,13 +11434,12 @@
       <c r="R49">
         <v>5.3683930000000002</v>
       </c>
-      <c r="U49" s="4" t="s">
+      <c r="U49" t="s">
         <v>103</v>
       </c>
-      <c r="V49" s="4">
+      <c r="V49">
         <v>45</v>
       </c>
-      <c r="W49" s="4"/>
     </row>
     <row r="50" spans="4:23">
       <c r="D50">
@@ -10803,13 +11448,13 @@
       <c r="E50">
         <v>34.357607000000002</v>
       </c>
-      <c r="K50" s="4" t="s">
+      <c r="K50" t="s">
         <v>99</v>
       </c>
-      <c r="L50" s="4">
+      <c r="L50">
         <v>18.961834148148149</v>
       </c>
-      <c r="M50" s="4">
+      <c r="M50">
         <v>28.455410500000006</v>
       </c>
       <c r="Q50">
@@ -10818,13 +11463,12 @@
       <c r="R50">
         <v>27.407136999999999</v>
       </c>
-      <c r="U50" s="4" t="s">
+      <c r="U50" t="s">
         <v>104</v>
       </c>
-      <c r="V50" s="4">
+      <c r="V50">
         <v>-2.5801872881105767</v>
       </c>
-      <c r="W50" s="4"/>
     </row>
     <row r="51" spans="4:23">
       <c r="D51">
@@ -10833,13 +11477,13 @@
       <c r="E51">
         <v>39.090671999999998</v>
       </c>
-      <c r="K51" s="4" t="s">
+      <c r="K51" t="s">
         <v>100</v>
       </c>
-      <c r="L51" s="4">
+      <c r="L51">
         <v>49.486806798110422</v>
       </c>
-      <c r="M51" s="4">
+      <c r="M51">
         <v>80.447471020117121</v>
       </c>
       <c r="Q51">
@@ -10848,13 +11492,12 @@
       <c r="R51">
         <v>30.938687999999999</v>
       </c>
-      <c r="U51" s="4" t="s">
+      <c r="U51" t="s">
         <v>105</v>
       </c>
-      <c r="V51" s="4">
+      <c r="V51">
         <v>6.6046553151036793E-3</v>
       </c>
-      <c r="W51" s="4"/>
     </row>
     <row r="52" spans="4:23">
       <c r="D52">
@@ -10863,13 +11506,13 @@
       <c r="E52">
         <v>30.456852999999999</v>
       </c>
-      <c r="K52" s="4" t="s">
+      <c r="K52" t="s">
         <v>101</v>
       </c>
-      <c r="L52" s="4">
+      <c r="L52">
         <v>9</v>
       </c>
-      <c r="M52" s="4">
+      <c r="M52">
         <v>10</v>
       </c>
       <c r="Q52">
@@ -10878,13 +11521,12 @@
       <c r="R52">
         <v>31.456980000000001</v>
       </c>
-      <c r="U52" s="4" t="s">
+      <c r="U52" t="s">
         <v>106</v>
       </c>
-      <c r="V52" s="4">
+      <c r="V52">
         <v>1.6794273926523535</v>
       </c>
-      <c r="W52" s="4"/>
     </row>
     <row r="53" spans="4:23">
       <c r="D53">
@@ -10893,54 +11535,51 @@
       <c r="E53">
         <v>38.751725</v>
       </c>
-      <c r="K53" s="4" t="s">
+      <c r="K53" t="s">
         <v>111</v>
       </c>
-      <c r="L53" s="4">
+      <c r="L53">
         <v>65.877746680349262</v>
       </c>
-      <c r="M53" s="4"/>
       <c r="Q53">
         <v>7.7812380000000001</v>
       </c>
       <c r="R53">
         <v>34.357607000000002</v>
       </c>
-      <c r="U53" s="4" t="s">
+      <c r="U53" t="s">
         <v>107</v>
       </c>
-      <c r="V53" s="4">
+      <c r="V53">
         <v>1.3209310630207359E-2</v>
       </c>
-      <c r="W53" s="4"/>
-    </row>
-    <row r="54" spans="4:23" ht="15" thickBot="1">
+    </row>
+    <row r="54" spans="4:23" ht="15.75" thickBot="1">
       <c r="D54">
         <v>22.615593000000001</v>
       </c>
       <c r="E54">
         <v>41.354227999999999</v>
       </c>
-      <c r="K54" s="4" t="s">
+      <c r="K54" t="s">
         <v>102</v>
       </c>
-      <c r="L54" s="4">
+      <c r="L54">
         <v>0</v>
       </c>
-      <c r="M54" s="4"/>
       <c r="Q54">
         <v>8.8605520000000002</v>
       </c>
       <c r="R54">
         <v>39.090671999999998</v>
       </c>
-      <c r="U54" s="5" t="s">
+      <c r="U54" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="V54" s="5">
+      <c r="V54" s="3">
         <v>2.0141033888808457</v>
       </c>
-      <c r="W54" s="5"/>
+      <c r="W54" s="3"/>
     </row>
     <row r="55" spans="4:23">
       <c r="D55">
@@ -10949,13 +11588,12 @@
       <c r="E55">
         <v>25.324967000000001</v>
       </c>
-      <c r="K55" s="4" t="s">
+      <c r="K55" t="s">
         <v>103</v>
       </c>
-      <c r="L55" s="4">
+      <c r="L55">
         <v>17</v>
       </c>
-      <c r="M55" s="4"/>
       <c r="Q55">
         <v>10.206614999999999</v>
       </c>
@@ -10970,13 +11608,12 @@
       <c r="E56">
         <v>24.631449</v>
       </c>
-      <c r="K56" s="4" t="s">
+      <c r="K56" t="s">
         <v>104</v>
       </c>
-      <c r="L56" s="4">
+      <c r="L56">
         <v>-2.5456865842639913</v>
       </c>
-      <c r="M56" s="4"/>
       <c r="Q56">
         <v>14.210526</v>
       </c>
@@ -10991,84 +11628,81 @@
       <c r="E57">
         <v>20.296095999999999</v>
       </c>
-      <c r="K57" s="4" t="s">
+      <c r="K57" t="s">
         <v>105</v>
       </c>
-      <c r="L57" s="4">
+      <c r="L57">
         <v>1.044721861867267E-2</v>
       </c>
-      <c r="M57" s="4"/>
       <c r="Q57">
         <v>26.940118999999999</v>
       </c>
       <c r="R57">
         <v>41.354227999999999</v>
       </c>
-      <c r="U57" s="8" t="s">
+      <c r="U57" s="6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="4:23" ht="15" thickBot="1">
-      <c r="K58" s="4" t="s">
+    <row r="58" spans="4:23" ht="15.75" thickBot="1">
+      <c r="K58" t="s">
         <v>106</v>
       </c>
-      <c r="L58" s="4">
+      <c r="L58">
         <v>1.7396067260750732</v>
       </c>
-      <c r="M58" s="4"/>
       <c r="Q58">
         <v>10.094481</v>
       </c>
       <c r="R58">
         <v>25.324967000000001</v>
       </c>
-      <c r="U58" s="7" t="s">
+      <c r="U58" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="59" spans="4:23">
-      <c r="K59" s="4" t="s">
+      <c r="K59" t="s">
         <v>107</v>
       </c>
-      <c r="L59" s="4">
+      <c r="L59">
         <v>2.089443723734534E-2</v>
       </c>
-      <c r="M59" s="4"/>
       <c r="Q59">
         <v>36.113652999999999</v>
       </c>
       <c r="R59">
         <v>24.631449</v>
       </c>
-      <c r="U59" s="6"/>
-      <c r="V59" s="6" t="s">
+      <c r="U59" s="4"/>
+      <c r="V59" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="W59" s="6" t="s">
+      <c r="W59" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="60" spans="4:23" ht="15" thickBot="1">
-      <c r="K60" s="5" t="s">
+    <row r="60" spans="4:23" ht="15.75" thickBot="1">
+      <c r="K60" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="L60" s="5">
+      <c r="L60" s="3">
         <v>2.109815577833317</v>
       </c>
-      <c r="M60" s="5"/>
+      <c r="M60" s="3"/>
       <c r="Q60">
         <v>14.655714</v>
       </c>
       <c r="R60">
         <v>20.296095999999999</v>
       </c>
-      <c r="U60" s="4" t="s">
+      <c r="U60" t="s">
         <v>99</v>
       </c>
-      <c r="V60" s="4">
+      <c r="V60">
         <v>18.961834148148146</v>
       </c>
-      <c r="W60" s="4">
+      <c r="W60">
         <v>28.455410499999999</v>
       </c>
     </row>
@@ -11076,13 +11710,13 @@
       <c r="Q61">
         <v>22.608398000000001</v>
       </c>
-      <c r="U61" s="4" t="s">
+      <c r="U61" t="s">
         <v>100</v>
       </c>
-      <c r="V61" s="4">
+      <c r="V61">
         <v>144.02790603704489</v>
       </c>
-      <c r="W61" s="4">
+      <c r="W61">
         <v>171.30275626533091</v>
       </c>
     </row>
@@ -11096,13 +11730,13 @@
       <c r="Q62">
         <v>58.124909000000002</v>
       </c>
-      <c r="U62" s="4" t="s">
+      <c r="U62" t="s">
         <v>101</v>
       </c>
-      <c r="V62" s="4">
+      <c r="V62">
         <v>27</v>
       </c>
-      <c r="W62" s="4">
+      <c r="W62">
         <v>20</v>
       </c>
     </row>
@@ -11116,13 +11750,12 @@
       <c r="Q63">
         <v>23.981276999999999</v>
       </c>
-      <c r="U63" s="4" t="s">
+      <c r="U63" t="s">
         <v>102</v>
       </c>
-      <c r="V63" s="4">
+      <c r="V63">
         <v>0</v>
       </c>
-      <c r="W63" s="4"/>
     </row>
     <row r="64" spans="4:23">
       <c r="D64">
@@ -11134,13 +11767,12 @@
       <c r="Q64">
         <v>6.4825799999999996</v>
       </c>
-      <c r="U64" s="4" t="s">
+      <c r="U64" t="s">
         <v>103</v>
       </c>
-      <c r="V64" s="4">
+      <c r="V64">
         <v>39</v>
       </c>
-      <c r="W64" s="4"/>
     </row>
     <row r="65" spans="4:23">
       <c r="D65">
@@ -11152,13 +11784,12 @@
       <c r="Q65">
         <v>7.4210529999999997</v>
       </c>
-      <c r="U65" s="4" t="s">
+      <c r="U65" t="s">
         <v>104</v>
       </c>
-      <c r="V65" s="4">
+      <c r="V65">
         <v>-2.5464208706143445</v>
       </c>
-      <c r="W65" s="4"/>
     </row>
     <row r="66" spans="4:23">
       <c r="D66">
@@ -11170,13 +11801,12 @@
       <c r="Q66">
         <v>34.287424999999999</v>
       </c>
-      <c r="U66" s="4" t="s">
+      <c r="U66" t="s">
         <v>105</v>
       </c>
-      <c r="V66" s="4">
+      <c r="V66">
         <v>7.4723988726281866E-3</v>
       </c>
-      <c r="W66" s="4"/>
     </row>
     <row r="67" spans="4:23">
       <c r="D67">
@@ -11188,13 +11818,12 @@
       <c r="Q67">
         <v>17.930986000000001</v>
       </c>
-      <c r="U67" s="4" t="s">
+      <c r="U67" t="s">
         <v>106</v>
       </c>
-      <c r="V67" s="4">
+      <c r="V67">
         <v>1.6848751217112248</v>
       </c>
-      <c r="W67" s="4"/>
     </row>
     <row r="68" spans="4:23">
       <c r="D68">
@@ -11203,28 +11832,27 @@
       <c r="E68">
         <v>41.354227999999999</v>
       </c>
-      <c r="U68" s="4" t="s">
+      <c r="U68" t="s">
         <v>107</v>
       </c>
-      <c r="V68" s="4">
+      <c r="V68">
         <v>1.4944797745256373E-2</v>
       </c>
-      <c r="W68" s="4"/>
-    </row>
-    <row r="69" spans="4:23" ht="15" thickBot="1">
+    </row>
+    <row r="69" spans="4:23" ht="15.75" thickBot="1">
       <c r="D69">
         <v>25.324967000000001</v>
       </c>
       <c r="E69">
         <v>60.294035000000001</v>
       </c>
-      <c r="U69" s="5" t="s">
+      <c r="U69" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="V69" s="5">
+      <c r="V69" s="3">
         <v>2.0226909200367595</v>
       </c>
-      <c r="W69" s="5"/>
+      <c r="W69" s="3"/>
     </row>
     <row r="70" spans="4:23">
       <c r="D70">
@@ -11271,391 +11899,219 @@
         <v>119</v>
       </c>
     </row>
-    <row r="77" spans="4:23" ht="15" thickBot="1"/>
+    <row r="77" spans="4:23" ht="15.75" thickBot="1"/>
     <row r="78" spans="4:23">
-      <c r="D78" s="10" t="s">
+      <c r="D78" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="E78" s="10"/>
+      <c r="E78" s="8"/>
     </row>
     <row r="79" spans="4:23">
-      <c r="D79" s="4" t="s">
+      <c r="D79" t="s">
         <v>121</v>
       </c>
-      <c r="E79" s="4">
+      <c r="E79">
         <v>0.37363996284209949</v>
       </c>
     </row>
     <row r="80" spans="4:23">
-      <c r="D80" s="4" t="s">
+      <c r="D80" t="s">
         <v>122</v>
       </c>
-      <c r="E80" s="4">
+      <c r="E80">
         <v>0.1396068218326455</v>
       </c>
     </row>
     <row r="81" spans="4:12">
-      <c r="D81" s="4" t="s">
+      <c r="D81" t="s">
         <v>123</v>
       </c>
-      <c r="E81" s="4">
+      <c r="E81">
         <v>3.2057674561726202E-2</v>
       </c>
     </row>
     <row r="82" spans="4:12">
-      <c r="D82" s="4" t="s">
+      <c r="D82" t="s">
         <v>124</v>
       </c>
-      <c r="E82" s="4">
+      <c r="E82">
         <v>11.387177956721336</v>
       </c>
     </row>
-    <row r="83" spans="4:12" ht="15" thickBot="1">
-      <c r="D83" s="5" t="s">
+    <row r="83" spans="4:12" ht="15.75" thickBot="1">
+      <c r="D83" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="E83" s="5">
+      <c r="E83" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="85" spans="4:12" ht="15" thickBot="1">
+    <row r="85" spans="4:12" ht="15.75" thickBot="1">
       <c r="D85" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="86" spans="4:12">
-      <c r="D86" s="6"/>
-      <c r="E86" s="6" t="s">
+      <c r="D86" s="4"/>
+      <c r="E86" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F86" s="6" t="s">
+      <c r="F86" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="G86" s="6" t="s">
+      <c r="G86" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="H86" s="6" t="s">
+      <c r="H86" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="I86" s="6" t="s">
+      <c r="I86" s="4" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="87" spans="4:12">
-      <c r="D87" s="4" t="s">
+      <c r="D87" t="s">
         <v>126</v>
       </c>
-      <c r="E87" s="4">
+      <c r="E87">
         <v>1</v>
       </c>
-      <c r="F87" s="4">
+      <c r="F87">
         <v>168.31851258083566</v>
       </c>
-      <c r="G87" s="4">
+      <c r="G87">
         <v>168.31851258083566</v>
       </c>
-      <c r="H87" s="4">
+      <c r="H87">
         <v>1.2980746512194283</v>
       </c>
-      <c r="I87" s="4">
+      <c r="I87">
         <v>0.28752818959490545</v>
       </c>
     </row>
     <row r="88" spans="4:12">
-      <c r="D88" s="4" t="s">
+      <c r="D88" t="s">
         <v>127</v>
       </c>
-      <c r="E88" s="4">
+      <c r="E88">
         <v>8</v>
       </c>
-      <c r="F88" s="4">
+      <c r="F88">
         <v>1037.3425745443226</v>
       </c>
-      <c r="G88" s="4">
+      <c r="G88">
         <v>129.66782181804032</v>
       </c>
-      <c r="H88" s="4"/>
-      <c r="I88" s="4"/>
-    </row>
-    <row r="89" spans="4:12" ht="15" thickBot="1">
-      <c r="D89" s="5" t="s">
+    </row>
+    <row r="89" spans="4:12" ht="15.75" thickBot="1">
+      <c r="D89" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E89" s="5">
+      <c r="E89" s="3">
         <v>9</v>
       </c>
-      <c r="F89" s="5">
+      <c r="F89" s="3">
         <v>1205.6610871251582</v>
       </c>
-      <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
-      <c r="I89" s="5"/>
-    </row>
-    <row r="90" spans="4:12" ht="15" thickBot="1"/>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
+      <c r="I89" s="3"/>
+    </row>
+    <row r="90" spans="4:12" ht="15.75" thickBot="1"/>
     <row r="91" spans="4:12">
-      <c r="D91" s="6"/>
-      <c r="E91" s="6" t="s">
+      <c r="D91" s="4"/>
+      <c r="E91" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="F91" s="6" t="s">
+      <c r="F91" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="G91" s="6" t="s">
+      <c r="G91" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="H91" s="6" t="s">
+      <c r="H91" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="I91" s="6" t="s">
+      <c r="I91" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="J91" s="6" t="s">
+      <c r="J91" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="K91" s="6" t="s">
+      <c r="K91" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="L91" s="6" t="s">
+      <c r="L91" s="4" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="92" spans="4:12">
-      <c r="D92" s="4" t="s">
+      <c r="D92" t="s">
         <v>129</v>
       </c>
-      <c r="E92" s="4">
+      <c r="E92">
         <v>5.4036584824827152</v>
       </c>
-      <c r="F92" s="4">
+      <c r="F92">
         <v>14.072654641634324</v>
       </c>
-      <c r="G92" s="4">
+      <c r="G92">
         <v>0.3839828817013563</v>
       </c>
-      <c r="H92" s="4">
+      <c r="H92">
         <v>0.71099559982347749</v>
       </c>
-      <c r="I92" s="4">
+      <c r="I92">
         <v>-27.047941314426151</v>
       </c>
-      <c r="J92" s="4">
+      <c r="J92">
         <v>37.855258279391578</v>
       </c>
-      <c r="K92" s="4">
+      <c r="K92">
         <v>-27.047941314426151</v>
       </c>
-      <c r="L92" s="4">
+      <c r="L92">
         <v>37.855258279391578</v>
       </c>
     </row>
-    <row r="93" spans="4:12" ht="15" thickBot="1">
-      <c r="D93" s="5" t="s">
+    <row r="93" spans="4:12" ht="15.75" thickBot="1">
+      <c r="D93" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="E93" s="5">
+      <c r="E93" s="3">
         <v>0.43045497313062059</v>
       </c>
-      <c r="F93" s="5">
+      <c r="F93" s="3">
         <v>0.3778138680598595</v>
       </c>
-      <c r="G93" s="5">
+      <c r="G93" s="3">
         <v>1.1393307909555634</v>
       </c>
-      <c r="H93" s="5">
+      <c r="H93" s="3">
         <v>0.28752818959490484</v>
       </c>
-      <c r="I93" s="5">
+      <c r="I93" s="3">
         <v>-0.44078536895289705</v>
       </c>
-      <c r="J93" s="5">
+      <c r="J93" s="3">
         <v>1.3016953152141382</v>
       </c>
-      <c r="K93" s="5">
+      <c r="K93" s="3">
         <v>-0.44078536895289705</v>
       </c>
-      <c r="L93" s="5">
+      <c r="L93" s="3">
         <v>1.3016953152141382</v>
       </c>
     </row>
-    <row r="96" spans="4:12">
-      <c r="D96" s="11"/>
-      <c r="E96" s="11"/>
-      <c r="F96" s="11"/>
-      <c r="G96" s="11"/>
-    </row>
-    <row r="97" spans="4:7">
-      <c r="D97" s="11"/>
-      <c r="E97" s="11"/>
-      <c r="F97" s="11"/>
-      <c r="G97" s="11"/>
-    </row>
-    <row r="98" spans="4:7">
-      <c r="D98" s="11"/>
-      <c r="E98" s="11"/>
-      <c r="F98" s="11"/>
-      <c r="G98" s="11"/>
-    </row>
-    <row r="99" spans="4:7">
-      <c r="D99" s="12"/>
-      <c r="E99" s="12"/>
-      <c r="F99" s="12"/>
-      <c r="G99" s="11"/>
-    </row>
-    <row r="100" spans="4:7">
-      <c r="D100" s="4"/>
-      <c r="E100" s="4"/>
-      <c r="F100" s="4"/>
-      <c r="G100" s="11"/>
-    </row>
-    <row r="101" spans="4:7">
-      <c r="D101" s="4"/>
-      <c r="E101" s="4"/>
-      <c r="F101" s="4"/>
-      <c r="G101" s="11"/>
-    </row>
-    <row r="102" spans="4:7">
-      <c r="D102" s="4"/>
-      <c r="E102" s="4"/>
-      <c r="F102" s="4"/>
-      <c r="G102" s="11"/>
-    </row>
-    <row r="103" spans="4:7">
-      <c r="D103" s="4"/>
-      <c r="E103" s="4"/>
-      <c r="F103" s="4"/>
-      <c r="G103" s="11"/>
-    </row>
-    <row r="104" spans="4:7">
-      <c r="D104" s="4"/>
-      <c r="E104" s="4"/>
-      <c r="F104" s="4"/>
-      <c r="G104" s="11"/>
-    </row>
-    <row r="105" spans="4:7">
-      <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
-      <c r="F105" s="4"/>
-      <c r="G105" s="11"/>
-    </row>
-    <row r="106" spans="4:7">
-      <c r="D106" s="4"/>
-      <c r="E106" s="4"/>
-      <c r="F106" s="4"/>
-      <c r="G106" s="11"/>
-    </row>
-    <row r="107" spans="4:7">
-      <c r="D107" s="4"/>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-      <c r="G107" s="11"/>
-    </row>
-    <row r="108" spans="4:7">
-      <c r="D108" s="4"/>
-      <c r="E108" s="4"/>
-      <c r="F108" s="4"/>
-      <c r="G108" s="11"/>
-    </row>
-    <row r="109" spans="4:7">
-      <c r="D109" s="4"/>
-      <c r="E109" s="4"/>
-      <c r="F109" s="4"/>
-      <c r="G109" s="11"/>
-    </row>
-    <row r="110" spans="4:7">
-      <c r="D110" s="11"/>
-      <c r="E110" s="11"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="11"/>
-    </row>
-    <row r="111" spans="4:7">
-      <c r="D111" s="11"/>
-      <c r="E111" s="11"/>
-      <c r="F111" s="11"/>
-      <c r="G111" s="11"/>
-    </row>
-    <row r="112" spans="4:7">
-      <c r="D112" s="11"/>
-      <c r="E112" s="11"/>
-      <c r="F112" s="11"/>
-      <c r="G112" s="11"/>
-    </row>
-    <row r="113" spans="4:7">
-      <c r="D113" s="11"/>
-      <c r="E113" s="11"/>
-      <c r="F113" s="11"/>
-      <c r="G113" s="11"/>
-    </row>
-    <row r="114" spans="4:7">
-      <c r="D114" s="11"/>
-      <c r="E114" s="11"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="11"/>
-    </row>
-    <row r="115" spans="4:7">
-      <c r="D115" s="11"/>
-      <c r="E115" s="11"/>
-      <c r="F115" s="11"/>
-      <c r="G115" s="11"/>
-    </row>
-    <row r="116" spans="4:7">
-      <c r="D116" s="12"/>
-      <c r="E116" s="12"/>
-      <c r="F116" s="12"/>
-      <c r="G116" s="11"/>
-    </row>
-    <row r="117" spans="4:7">
-      <c r="D117" s="4"/>
-      <c r="E117" s="4"/>
-      <c r="F117" s="4"/>
-      <c r="G117" s="11"/>
-    </row>
-    <row r="118" spans="4:7">
-      <c r="D118" s="4"/>
-      <c r="E118" s="4"/>
-      <c r="F118" s="4"/>
-      <c r="G118" s="11"/>
-    </row>
-    <row r="119" spans="4:7">
-      <c r="D119" s="4"/>
-      <c r="E119" s="4"/>
-      <c r="F119" s="4"/>
-      <c r="G119" s="11"/>
-    </row>
-    <row r="120" spans="4:7">
-      <c r="D120" s="4"/>
-      <c r="E120" s="4"/>
-      <c r="F120" s="4"/>
-      <c r="G120" s="11"/>
-    </row>
-    <row r="121" spans="4:7">
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
-      <c r="G121" s="11"/>
-    </row>
-    <row r="122" spans="4:7">
-      <c r="D122" s="4"/>
-      <c r="E122" s="4"/>
-      <c r="F122" s="4"/>
-      <c r="G122" s="11"/>
-    </row>
-    <row r="123" spans="4:7">
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
-      <c r="F123" s="4"/>
-      <c r="G123" s="11"/>
-    </row>
-    <row r="124" spans="4:7">
-      <c r="D124" s="11"/>
-      <c r="E124" s="11"/>
-      <c r="F124" s="11"/>
-      <c r="G124" s="11"/>
-    </row>
-    <row r="125" spans="4:7">
-      <c r="D125" s="11"/>
-      <c r="E125" s="11"/>
-      <c r="F125" s="11"/>
-      <c r="G125" s="11"/>
+    <row r="99" spans="4:6">
+      <c r="D99" s="9"/>
+      <c r="E99" s="9"/>
+      <c r="F99" s="9"/>
+    </row>
+    <row r="116" spans="4:6">
+      <c r="D116" s="9"/>
+      <c r="E116" s="9"/>
+      <c r="F116" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11665,4 +12121,317 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02490D31-8144-4D02-A37F-D0BDE3454DA1}">
+  <dimension ref="D3:L34"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="3" spans="4:6">
+      <c r="D3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="4:6">
+      <c r="D4" s="2">
+        <v>0.147929</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.49503999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="4:6">
+      <c r="D5" s="2">
+        <v>0.85066200000000003</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.59295100000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="4:6">
+      <c r="D6" s="2">
+        <v>0.88</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.25284800000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="4:6">
+      <c r="D7" s="2">
+        <v>0.921269</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.39312900000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="4:6">
+      <c r="D8" s="2">
+        <v>0.60075999999999996</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.43397799999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="4:6">
+      <c r="D9" s="2">
+        <v>0.49684200000000001</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0.352771</v>
+      </c>
+    </row>
+    <row r="10" spans="4:6">
+      <c r="D10" s="2">
+        <v>0.67821100000000001</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.44958799999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="4:6">
+      <c r="D11" s="2">
+        <v>0.58125499999999997</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.63485400000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="4:6">
+      <c r="D12" s="2">
+        <v>0.30175400000000002</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.46416099999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="4:6">
+      <c r="D13" s="2">
+        <v>0.67080700000000004</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+    </row>
+    <row r="16" spans="4:6">
+      <c r="D16" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="4:12" ht="15.75" thickBot="1"/>
+    <row r="18" spans="4:12">
+      <c r="D18" s="13"/>
+      <c r="E18" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+    </row>
+    <row r="19" spans="4:12">
+      <c r="D19" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="11">
+        <v>0.61294889999999991</v>
+      </c>
+      <c r="F19" s="11">
+        <v>0.45214666666666659</v>
+      </c>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+    </row>
+    <row r="20" spans="4:12">
+      <c r="D20" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="11">
+        <v>6.2023494600988945E-2</v>
+      </c>
+      <c r="F20" s="11">
+        <v>1.3575903256500044E-2</v>
+      </c>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+    </row>
+    <row r="21" spans="4:12">
+      <c r="D21" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="11">
+        <v>10</v>
+      </c>
+      <c r="F21" s="11">
+        <v>9</v>
+      </c>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14"/>
+    </row>
+    <row r="22" spans="4:12">
+      <c r="D22" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" s="11">
+        <v>3.9224628085935347E-2</v>
+      </c>
+      <c r="F22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+    </row>
+    <row r="23" spans="4:12">
+      <c r="D23" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E23" s="11">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="14"/>
+    </row>
+    <row r="24" spans="4:12">
+      <c r="D24" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E24" s="11">
+        <v>17</v>
+      </c>
+      <c r="F24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
+    </row>
+    <row r="25" spans="4:12">
+      <c r="D25" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" s="11">
+        <v>1.7670836690454677</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14"/>
+    </row>
+    <row r="26" spans="4:12">
+      <c r="D26" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" s="11">
+        <v>4.758001301771498E-2</v>
+      </c>
+      <c r="F26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14"/>
+    </row>
+    <row r="27" spans="4:12">
+      <c r="D27" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27" s="11">
+        <v>1.7396067260750732</v>
+      </c>
+      <c r="F27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14"/>
+    </row>
+    <row r="28" spans="4:12">
+      <c r="D28" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="E28" s="11">
+        <v>9.5160026035429959E-2</v>
+      </c>
+      <c r="F28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+    </row>
+    <row r="29" spans="4:12" ht="15.75" thickBot="1">
+      <c r="D29" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="12">
+        <v>2.109815577833317</v>
+      </c>
+      <c r="F29" s="12"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="14"/>
+    </row>
+    <row r="30" spans="4:12">
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
+    </row>
+    <row r="31" spans="4:12">
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+    </row>
+    <row r="32" spans="4:12">
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
+    </row>
+    <row r="33" spans="8:12">
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+    </row>
+    <row r="34" spans="8:12">
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added work on the group blink async in ms
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,24 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB40E47-D377-4711-B6D3-9B86D6CBF8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6725371-C27E-4A70-A4B5-6240CA480AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="165" yWindow="240" windowWidth="28635" windowHeight="15240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="BlinkRateMinute" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">Sheet2!$D$3</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">Sheet2!$D$4:$D$13</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Sheet3!$C$3</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Sheet3!$C$4:$C$13</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$E$3</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$E$4:$E$13</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$D$3</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet2!$D$4:$D$13</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet2!$E$3</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet2!$E$4:$E$13</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet3!$B$3</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet3!$B$4:$B$13</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet3!$C$3</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet3!$C$4:$C$13</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Sheet3!$B$3</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Sheet3!$B$4:$B$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="150">
   <si>
     <t>Group</t>
   </si>
@@ -477,6 +482,27 @@
   </si>
   <si>
     <t>Triad</t>
+  </si>
+  <si>
+    <t>2024 05 07 - triad S1 G2</t>
+  </si>
+  <si>
+    <t>2024 05 07 - triad S1 G4</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_11_04_Seminar_Mun_Session_1_Group_1</t>
+  </si>
+  <si>
+    <t>DYAD_2024_11_04_Seminar_Mun_Session_1_Group_2</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_11_11_Seminar_Mun_Session_1_Group_1</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_11_18_Seminar_Mun_Session_1_Group_1</t>
+  </si>
+  <si>
+    <t>Triads</t>
   </si>
 </sst>
 </file>
@@ -519,7 +545,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,6 +555,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -565,7 +597,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -596,6 +628,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4499,7 +4533,6 @@
     </cx:data>
   </cx:chartData>
   <cx:chart>
-    <cx:title pos="t" align="ctr" overlay="0"/>
     <cx:plotArea>
       <cx:plotAreaRegion>
         <cx:series layoutId="boxWhisker" uniqueId="{5F5FEFE0-8F79-4C9C-BDD4-A3321F378915}">
@@ -4535,6 +4568,127 @@
           </cx:layoutPr>
         </cx:series>
       </cx:plotAreaRegion>
+      <cx:axis id="0" hidden="1">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Synchronised Blinks (%)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+                </a:rPr>
+                <a:t>Synchronised Blinks (%)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="r" align="min" overlay="1"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.5</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.7</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>The mean blink asynchrony (ms) between the onset time of blinks of partners</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>The mean blink asynchrony (ms) between the onset time of blinks of partners</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{A5B4DEED-1E68-4B6B-87B2-059879358505}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.4</cx:f>
+              <cx:v>Dyads</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:noFill/>
+          </cx:spPr>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="1" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{BE8BCE1F-0F62-4B06-9656-6717B23429AD}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.6</cx:f>
+              <cx:v>Triads</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:noFill/>
+          </cx:spPr>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="1" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="1"/>
         <cx:tickLabels/>
@@ -4545,11 +4699,52 @@
         <cx:tickLabels/>
       </cx:axis>
     </cx:plotArea>
+    <cx:legend pos="r" align="min" overlay="1"/>
   </cx:chart>
 </cx:chartSpace>
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5425,6 +5620,521 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -9859,16 +10569,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>471487</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>115887</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>166687</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>420687</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>146050</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -9904,8 +10614,91 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="4738687" y="200025"/>
-              <a:ext cx="4572000" cy="2752725"/>
+              <a:off x="5602287" y="1539875"/>
+              <a:ext cx="4572000" cy="2663825"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-GB" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>530225</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F21AFA72-F260-644B-8F00-F76B6A97F61C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2359025" y="1073150"/>
+              <a:ext cx="4435475" cy="3251200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -10241,14 +11034,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.5703125" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="1" max="1" width="54.54296875" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -10700,6 +11493,36 @@
       </c>
       <c r="G26" t="s">
         <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -10710,13 +11533,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08CBB891-F584-4F5A-A553-41469C7D6F94}">
   <dimension ref="C1:AA116"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="57.140625" customWidth="1"/>
+    <col min="3" max="3" width="57.1796875" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="9" max="9" width="58.28515625" customWidth="1"/>
+    <col min="9" max="9" width="58.26953125" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="15" width="11.85546875" customWidth="1"/>
+    <col min="14" max="15" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:16">
@@ -11170,7 +11993,7 @@
         <v>-7.203443722093221E-2</v>
       </c>
     </row>
-    <row r="23" spans="11:27" ht="15.75" thickBot="1"/>
+    <row r="23" spans="11:27" ht="15" thickBot="1"/>
     <row r="24" spans="11:27">
       <c r="Y24" s="4"/>
       <c r="Z24" s="4"/>
@@ -11181,7 +12004,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="4:27" ht="15.75" thickBot="1">
+    <row r="33" spans="4:27" ht="15" thickBot="1">
       <c r="K33" s="5" t="s">
         <v>115</v>
       </c>
@@ -11195,7 +12018,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="4:27" ht="15.75" thickBot="1">
+    <row r="35" spans="4:27" ht="15" thickBot="1">
       <c r="K35" t="s">
         <v>99</v>
       </c>
@@ -11278,7 +12101,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="4:27" ht="15.75" thickBot="1">
+    <row r="42" spans="4:27" ht="15" thickBot="1">
       <c r="K42" t="s">
         <v>106</v>
       </c>
@@ -11316,7 +12139,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="4:27" ht="15.75" thickBot="1">
+    <row r="44" spans="4:27" ht="15" thickBot="1">
       <c r="K44" s="3" t="s">
         <v>108</v>
       </c>
@@ -11391,7 +12214,7 @@
         <v>155.54395391121008</v>
       </c>
     </row>
-    <row r="48" spans="4:27" ht="15.75" thickBot="1">
+    <row r="48" spans="4:27" ht="15" thickBot="1">
       <c r="D48">
         <v>2.4711409999999998</v>
       </c>
@@ -11554,7 +12377,7 @@
         <v>1.3209310630207359E-2</v>
       </c>
     </row>
-    <row r="54" spans="4:23" ht="15.75" thickBot="1">
+    <row r="54" spans="4:23" ht="15" thickBot="1">
       <c r="D54">
         <v>22.615593000000001</v>
       </c>
@@ -11644,7 +12467,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="4:23" ht="15.75" thickBot="1">
+    <row r="58" spans="4:23" ht="15" thickBot="1">
       <c r="K58" t="s">
         <v>106</v>
       </c>
@@ -11662,10 +12485,10 @@
       </c>
     </row>
     <row r="59" spans="4:23">
-      <c r="K59" t="s">
+      <c r="K59" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="L59">
+      <c r="L59" s="17">
         <v>2.089443723734534E-2</v>
       </c>
       <c r="Q59">
@@ -11682,7 +12505,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="60" spans="4:23" ht="15.75" thickBot="1">
+    <row r="60" spans="4:23" ht="15" thickBot="1">
       <c r="K60" s="3" t="s">
         <v>108</v>
       </c>
@@ -11839,7 +12662,7 @@
         <v>1.4944797745256373E-2</v>
       </c>
     </row>
-    <row r="69" spans="4:23" ht="15.75" thickBot="1">
+    <row r="69" spans="4:23" ht="15" thickBot="1">
       <c r="D69">
         <v>25.324967000000001</v>
       </c>
@@ -11899,7 +12722,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="77" spans="4:23" ht="15.75" thickBot="1"/>
+    <row r="77" spans="4:23" ht="15" thickBot="1"/>
     <row r="78" spans="4:23">
       <c r="D78" s="8" t="s">
         <v>120</v>
@@ -11938,7 +12761,7 @@
         <v>11.387177956721336</v>
       </c>
     </row>
-    <row r="83" spans="4:12" ht="15.75" thickBot="1">
+    <row r="83" spans="4:12" ht="15" thickBot="1">
       <c r="D83" s="3" t="s">
         <v>101</v>
       </c>
@@ -11946,7 +12769,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" spans="4:12" ht="15.75" thickBot="1">
+    <row r="85" spans="4:12" ht="15" thickBot="1">
       <c r="D85" t="s">
         <v>125</v>
       </c>
@@ -12003,7 +12826,7 @@
         <v>129.66782181804032</v>
       </c>
     </row>
-    <row r="89" spans="4:12" ht="15.75" thickBot="1">
+    <row r="89" spans="4:12" ht="15" thickBot="1">
       <c r="D89" s="3" t="s">
         <v>128</v>
       </c>
@@ -12017,7 +12840,7 @@
       <c r="H89" s="3"/>
       <c r="I89" s="3"/>
     </row>
-    <row r="90" spans="4:12" ht="15.75" thickBot="1"/>
+    <row r="90" spans="4:12" ht="15" thickBot="1"/>
     <row r="91" spans="4:12">
       <c r="D91" s="4"/>
       <c r="E91" s="4" t="s">
@@ -12074,7 +12897,7 @@
         <v>37.855258279391578</v>
       </c>
     </row>
-    <row r="93" spans="4:12" ht="15.75" thickBot="1">
+    <row r="93" spans="4:12" ht="15" thickBot="1">
       <c r="D93" s="3" t="s">
         <v>140</v>
       </c>
@@ -12125,8 +12948,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02490D31-8144-4D02-A37F-D0BDE3454DA1}">
-  <dimension ref="D3:L34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="C3:K47"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="3" spans="4:6">
       <c r="D3" t="s">
@@ -12220,218 +13043,510 @@
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="4:12" ht="15.75" thickBot="1"/>
-    <row r="18" spans="4:12">
-      <c r="D18" s="13"/>
-      <c r="E18" s="13" t="s">
+    <row r="17" spans="3:11" ht="15" thickBot="1"/>
+    <row r="18" spans="3:11">
+      <c r="D18" s="4"/>
+      <c r="E18" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-    </row>
-    <row r="19" spans="4:12">
-      <c r="D19" s="11" t="s">
+    </row>
+    <row r="19" spans="3:11">
+      <c r="D19" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19">
         <v>0.61294889999999991</v>
       </c>
-      <c r="F19" s="11">
+      <c r="F19">
         <v>0.45214666666666659</v>
       </c>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-    </row>
-    <row r="20" spans="4:12">
-      <c r="D20" s="11" t="s">
+    </row>
+    <row r="20" spans="3:11">
+      <c r="D20" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20">
         <v>6.2023494600988945E-2</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20">
         <v>1.3575903256500044E-2</v>
       </c>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-    </row>
-    <row r="21" spans="4:12">
-      <c r="D21" s="11" t="s">
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+    </row>
+    <row r="21" spans="3:11">
+      <c r="D21" t="s">
         <v>101</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21">
         <v>10</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21">
         <v>9</v>
       </c>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-    </row>
-    <row r="22" spans="4:12">
-      <c r="D22" s="11" t="s">
+    </row>
+    <row r="22" spans="3:11">
+      <c r="D22" t="s">
         <v>111</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22">
         <v>3.9224628085935347E-2</v>
       </c>
-      <c r="F22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-    </row>
-    <row r="23" spans="4:12">
-      <c r="D23" s="11" t="s">
+    </row>
+    <row r="23" spans="3:11">
+      <c r="D23" t="s">
         <v>102</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23">
         <v>0</v>
       </c>
-      <c r="F23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-    </row>
-    <row r="24" spans="4:12">
-      <c r="D24" s="11" t="s">
+    </row>
+    <row r="24" spans="3:11">
+      <c r="D24" t="s">
         <v>103</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24">
         <v>17</v>
       </c>
-      <c r="F24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-    </row>
-    <row r="25" spans="4:12">
-      <c r="D25" s="11" t="s">
+    </row>
+    <row r="25" spans="3:11">
+      <c r="D25" t="s">
         <v>104</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25">
         <v>1.7670836690454677</v>
       </c>
-      <c r="F25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-    </row>
-    <row r="26" spans="4:12">
-      <c r="D26" s="11" t="s">
+    </row>
+    <row r="26" spans="3:11">
+      <c r="D26" t="s">
         <v>105</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26">
         <v>4.758001301771498E-2</v>
       </c>
-      <c r="F26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
-    </row>
-    <row r="27" spans="4:12">
-      <c r="D27" s="11" t="s">
+    </row>
+    <row r="27" spans="3:11">
+      <c r="D27" t="s">
         <v>106</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27">
         <v>1.7396067260750732</v>
       </c>
-      <c r="F27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="14"/>
-    </row>
-    <row r="28" spans="4:12">
-      <c r="D28" s="11" t="s">
+    </row>
+    <row r="28" spans="3:11">
+      <c r="D28" t="s">
         <v>107</v>
       </c>
-      <c r="E28" s="11">
+      <c r="E28">
         <v>9.5160026035429959E-2</v>
       </c>
-      <c r="F28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="14"/>
-    </row>
-    <row r="29" spans="4:12" ht="15.75" thickBot="1">
-      <c r="D29" s="12" t="s">
+    </row>
+    <row r="29" spans="3:11" ht="15" thickBot="1">
+      <c r="D29" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="3">
         <v>2.109815577833317</v>
       </c>
-      <c r="F29" s="12"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-    </row>
-    <row r="30" spans="4:12">
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-    </row>
-    <row r="31" spans="4:12">
+      <c r="F29" s="3"/>
+    </row>
+    <row r="31" spans="3:11">
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
       <c r="H31" s="14"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-    </row>
-    <row r="32" spans="4:12">
+    </row>
+    <row r="32" spans="3:11">
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
       <c r="H32" s="14"/>
       <c r="I32" s="14"/>
       <c r="J32" s="14"/>
       <c r="K32" s="14"/>
-      <c r="L32" s="14"/>
-    </row>
-    <row r="33" spans="8:12">
+    </row>
+    <row r="33" spans="3:11">
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
       <c r="H33" s="14"/>
       <c r="I33" s="14"/>
       <c r="J33" s="14"/>
       <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-    </row>
-    <row r="34" spans="8:12">
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
+    </row>
+    <row r="34" spans="3:11">
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
       <c r="J34" s="14"/>
       <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
+    </row>
+    <row r="35" spans="3:11">
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+    </row>
+    <row r="36" spans="3:11">
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+    </row>
+    <row r="37" spans="3:11">
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
+    </row>
+    <row r="38" spans="3:11">
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14"/>
+    </row>
+    <row r="39" spans="3:11">
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="14"/>
+    </row>
+    <row r="40" spans="3:11">
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
+    </row>
+    <row r="41" spans="3:11">
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="14"/>
+    </row>
+    <row r="42" spans="3:11">
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+    </row>
+    <row r="43" spans="3:11">
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11"/>
+      <c r="I43" s="11"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+    </row>
+    <row r="44" spans="3:11">
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="14"/>
+    </row>
+    <row r="45" spans="3:11">
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+    </row>
+    <row r="46" spans="3:11">
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
+    </row>
+    <row r="47" spans="3:11">
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFC0AEBE-0304-40C9-AD55-B102AE5944DF}">
+  <dimension ref="B3:P20"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="3" spans="2:16">
+      <c r="B3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16">
+      <c r="B4">
+        <v>594.36</v>
+      </c>
+      <c r="C4">
+        <v>464.69001100000003</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16">
+      <c r="B5">
+        <v>501.77777800000001</v>
+      </c>
+      <c r="C5">
+        <v>583.26539500000001</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16">
+      <c r="B6">
+        <v>528.82102299999997</v>
+      </c>
+      <c r="C6">
+        <v>657.174126</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16">
+      <c r="B7">
+        <v>466.16581600000001</v>
+      </c>
+      <c r="C7">
+        <v>438.32892800000002</v>
+      </c>
+      <c r="N7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" ht="15" thickBot="1">
+      <c r="B8">
+        <v>592.886076</v>
+      </c>
+      <c r="C8">
+        <v>615.38994200000002</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16">
+      <c r="B9">
+        <v>479.042373</v>
+      </c>
+      <c r="C9">
+        <v>791.38082399999996</v>
+      </c>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="P9" s="13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16">
+      <c r="B10">
+        <v>477.22127699999999</v>
+      </c>
+      <c r="C10">
+        <v>695.81287599999996</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O10" s="11">
+        <v>500.27759300000008</v>
+      </c>
+      <c r="P10" s="11">
+        <v>594.43553344444445</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16">
+      <c r="B11">
+        <v>331.89349099999998</v>
+      </c>
+      <c r="C11">
+        <v>527.410031</v>
+      </c>
+      <c r="N11" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="O11" s="11">
+        <v>5555.4812917667441</v>
+      </c>
+      <c r="P11" s="11">
+        <v>12447.904788325191</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16">
+      <c r="B12">
+        <v>535.348837</v>
+      </c>
+      <c r="C12">
+        <v>576.467668</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="O12" s="11">
+        <v>10</v>
+      </c>
+      <c r="P12" s="11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16">
+      <c r="B13">
+        <v>495.25925899999999</v>
+      </c>
+      <c r="N13" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="O13" s="11">
+        <v>8798.974701911895</v>
+      </c>
+      <c r="P13" s="11"/>
+    </row>
+    <row r="14" spans="2:16">
+      <c r="N14" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="O14" s="11">
+        <v>0</v>
+      </c>
+      <c r="P14" s="11"/>
+    </row>
+    <row r="15" spans="2:16">
+      <c r="N15" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="O15" s="11">
+        <v>17</v>
+      </c>
+      <c r="P15" s="11"/>
+    </row>
+    <row r="16" spans="2:16">
+      <c r="N16" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="O16" s="11">
+        <v>-2.1846676115030039</v>
+      </c>
+      <c r="P16" s="11"/>
+    </row>
+    <row r="17" spans="14:16">
+      <c r="N17" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="O17" s="11">
+        <v>2.1603458578222112E-2</v>
+      </c>
+      <c r="P17" s="11"/>
+    </row>
+    <row r="18" spans="14:16">
+      <c r="N18" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="O18" s="11">
+        <v>1.7396067260750732</v>
+      </c>
+      <c r="P18" s="11"/>
+    </row>
+    <row r="19" spans="14:16">
+      <c r="N19" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="O19" s="16">
+        <v>4.3206917156444223E-2</v>
+      </c>
+      <c r="P19" s="11"/>
+    </row>
+    <row r="20" spans="14:16" ht="15" thickBot="1">
+      <c r="N20" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="O20" s="12">
+        <v>2.109815577833317</v>
+      </c>
+      <c r="P20" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
small changes to include negative delta time from sync binks
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6725371-C27E-4A70-A4B5-6240CA480AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380B2009-E563-432D-9C2E-3F49BF5D4D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="603" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,18 +19,20 @@
     <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet2!$D$3</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet2!$D$4:$D$13</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">Sheet3!$C$3</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">Sheet3!$C$4:$C$13</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$E$3</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$E$4:$E$13</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet3!$B$3</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet3!$B$4:$B$13</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet3!$C$3</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet3!$C$4:$C$13</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Sheet3!$B$3</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Sheet3!$B$4:$B$13</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">BlinkRateMinute!$F$2:$F$11</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">BlinkRateMinute!$P$2:$P$10</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Sheet3!$B$3</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Sheet3!$B$4:$B$13</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Sheet3!$C$3</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Sheet3!$C$4:$C$13</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$D$3</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$D$4:$D$13</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$E$3</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet2!$E$4:$E$13</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet3!$B$3</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet3!$B$4:$B$13</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Sheet3!$C$3</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Sheet3!$C$4:$C$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -597,7 +599,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -619,16 +621,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4122,6 +4114,36 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Dyads Blink Rate per</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> Minute (BPM)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4213,9 +4235,39 @@
               <c:layout>
                 <c:manualLayout>
                   <c:x val="-3.6110017497812771E-2"/>
-                  <c:y val="-3.6596522995601156E-2"/>
+                  <c:y val="-7.8691147588244831E-2"/>
                 </c:manualLayout>
               </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US"/>
+                      <a:t>r=0.036</a:t>
+                    </a:r>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>  p=.28</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -4363,6 +4415,68 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>BPM Participant 2</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -4425,6 +4539,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>BPM Participant 1</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -4523,22 +4692,169 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
   <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Dyads vs Triads on BPM</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Dyads vs Triads on BPM</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{4DFF839D-C16C-4082-A573-2E00517ECB81}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Dyads BPM</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:noFill/>
+          </cx:spPr>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="1" outliers="0"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000001-722A-435E-990A-4B385DA554D8}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Triads BPM</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:noFill/>
+          </cx:spPr>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" outliers="0"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0" hidden="1">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Blink Rate per Minute (BPM)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+                </a:rPr>
+                <a:t>Blink Rate per Minute (BPM)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="r" align="min" overlay="1"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.3</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.5</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Synced Blink % on Dyads vs Triads</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Synced Blink % on Dyads vs Triads</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
         <cx:series layoutId="boxWhisker" uniqueId="{5F5FEFE0-8F79-4C9C-BDD4-A3321F378915}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.0</cx:f>
+              <cx:f>_xlchart.v1.2</cx:f>
               <cx:v>Dyad</cx:v>
             </cx:txData>
           </cx:tx>
@@ -4554,7 +4870,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{3BB713B9-C79C-4E48-A5E2-750F24D24DB1}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.2</cx:f>
+              <cx:f>_xlchart.v1.4</cx:f>
               <cx:v>Triad</cx:v>
             </cx:txData>
           </cx:tx>
@@ -4611,17 +4927,17 @@
 </cx:chartSpace>
 </file>
 
-<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chartEx3.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.5</cx:f>
+        <cx:f>_xlchart.v1.7</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.7</cx:f>
+        <cx:f>_xlchart.v1.9</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -4659,7 +4975,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{A5B4DEED-1E68-4B6B-87B2-059879358505}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.4</cx:f>
+              <cx:f>_xlchart.v1.6</cx:f>
               <cx:v>Dyads</cx:v>
             </cx:txData>
           </cx:tx>
@@ -4675,7 +4991,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{BE8BCE1F-0F62-4B06-9656-6717B23429AD}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.6</cx:f>
+              <cx:f>_xlchart.v1.8</cx:f>
               <cx:v>Triads</cx:v>
             </cx:txData>
           </cx:tx>
@@ -4689,12 +5005,40 @@
           </cx:layoutPr>
         </cx:series>
       </cx:plotAreaRegion>
-      <cx:axis id="0">
+      <cx:axis id="0" hidden="1">
         <cx:catScaling gapWidth="1"/>
         <cx:tickLabels/>
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Miliseconds (ms)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+                </a:rPr>
+                <a:t>Miliseconds (ms)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
@@ -4745,6 +5089,46 @@
 </file>
 
 <file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors11.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -6135,6 +6519,521 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -10562,6 +11461,213 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>164354</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>32871</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>328706</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>153894</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="9" name="Chart 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28F7F133-3464-1E1E-94CD-EEDE7FAACFD7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="12819530" y="11679518"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-GB" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>250657</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>122676</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>391613</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>43446</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Right Bracket 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D671B8F-F4F1-0352-0E3F-675216A0B0D0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="15171290" y="13319175"/>
+          <a:ext cx="104585" cy="1050009"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightBracket">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:schemeClr val="bg2">
+              <a:lumMod val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-GB" sz="1100" kern="1200"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>645026</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>3342</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="254942" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="TextBox 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28EAECF1-FDD5-F787-531E-8A8E9BEC9249}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15092947" y="13856368"/>
+          <a:ext cx="254942" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>*</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -10652,16 +11758,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>530225</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>269875</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -10697,7 +11803,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="2359025" y="1073150"/>
+              <a:off x="2708275" y="685800"/>
               <a:ext cx="4435475" cy="3251200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -10728,6 +11834,135 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>359103</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>166414</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>96345</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>74453</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Right Bracket 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{991DCF15-4252-48FA-9A77-51DD0CF16698}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="5051532" y="2870640"/>
+          <a:ext cx="91970" cy="954690"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightBracket">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:schemeClr val="bg2">
+              <a:lumMod val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-GB" sz="1100" kern="1200"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>79059</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>50092</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="254942" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3CD88C7-C5D2-49B6-9613-D694FF38EC3F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4948852" y="3369609"/>
+          <a:ext cx="254942" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>*</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -12485,11 +13720,11 @@
       </c>
     </row>
     <row r="59" spans="4:23">
-      <c r="K59" s="17" t="s">
+      <c r="K59" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="L59" s="17">
-        <v>2.089443723734534E-2</v>
+      <c r="L59" s="11">
+        <v>2.0894437237345301E-2</v>
       </c>
       <c r="Q59">
         <v>36.113652999999999</v>
@@ -12948,7 +14183,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02490D31-8144-4D02-A37F-D0BDE3454DA1}">
-  <dimension ref="C3:K47"/>
+  <dimension ref="D3:J34"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="3" spans="4:6">
@@ -13043,8 +14278,8 @@
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="3:11" ht="15" thickBot="1"/>
-    <row r="18" spans="3:11">
+    <row r="17" spans="4:10" ht="15" thickBot="1"/>
+    <row r="18" spans="4:10">
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
         <v>97</v>
@@ -13053,7 +14288,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="3:11">
+    <row r="19" spans="4:10">
       <c r="D19" t="s">
         <v>99</v>
       </c>
@@ -13064,7 +14299,7 @@
         <v>0.45214666666666659</v>
       </c>
     </row>
-    <row r="20" spans="3:11">
+    <row r="20" spans="4:10">
       <c r="D20" t="s">
         <v>100</v>
       </c>
@@ -13078,7 +14313,7 @@
       <c r="I20" s="9"/>
       <c r="J20" s="9"/>
     </row>
-    <row r="21" spans="3:11">
+    <row r="21" spans="4:10">
       <c r="D21" t="s">
         <v>101</v>
       </c>
@@ -13089,7 +14324,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="3:11">
+    <row r="22" spans="4:10">
       <c r="D22" t="s">
         <v>111</v>
       </c>
@@ -13097,7 +14332,7 @@
         <v>3.9224628085935347E-2</v>
       </c>
     </row>
-    <row r="23" spans="3:11">
+    <row r="23" spans="4:10">
       <c r="D23" t="s">
         <v>102</v>
       </c>
@@ -13105,7 +14340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:11">
+    <row r="24" spans="4:10">
       <c r="D24" t="s">
         <v>103</v>
       </c>
@@ -13113,7 +14348,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="3:11">
+    <row r="25" spans="4:10">
       <c r="D25" t="s">
         <v>104</v>
       </c>
@@ -13121,7 +14356,7 @@
         <v>1.7670836690454677</v>
       </c>
     </row>
-    <row r="26" spans="3:11">
+    <row r="26" spans="4:10">
       <c r="D26" t="s">
         <v>105</v>
       </c>
@@ -13129,7 +14364,7 @@
         <v>4.758001301771498E-2</v>
       </c>
     </row>
-    <row r="27" spans="3:11">
+    <row r="27" spans="4:10">
       <c r="D27" t="s">
         <v>106</v>
       </c>
@@ -13137,7 +14372,7 @@
         <v>1.7396067260750732</v>
       </c>
     </row>
-    <row r="28" spans="3:11">
+    <row r="28" spans="4:10">
       <c r="D28" t="s">
         <v>107</v>
       </c>
@@ -13145,7 +14380,7 @@
         <v>9.5160026035429959E-2</v>
       </c>
     </row>
-    <row r="29" spans="3:11" ht="15" thickBot="1">
+    <row r="29" spans="4:10" ht="15" thickBot="1">
       <c r="D29" s="3" t="s">
         <v>108</v>
       </c>
@@ -13154,192 +14389,10 @@
       </c>
       <c r="F29" s="3"/>
     </row>
-    <row r="31" spans="3:11">
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-    </row>
-    <row r="32" spans="3:11">
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
-    </row>
-    <row r="33" spans="3:11">
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-    </row>
-    <row r="34" spans="3:11">
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="14"/>
-    </row>
-    <row r="35" spans="3:11">
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="14"/>
-      <c r="K35" s="14"/>
-    </row>
-    <row r="36" spans="3:11">
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="14"/>
-      <c r="K36" s="14"/>
-    </row>
-    <row r="37" spans="3:11">
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="14"/>
-      <c r="K37" s="14"/>
-    </row>
-    <row r="38" spans="3:11">
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="14"/>
-      <c r="K38" s="14"/>
-    </row>
-    <row r="39" spans="3:11">
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="14"/>
-      <c r="K39" s="14"/>
-    </row>
-    <row r="40" spans="3:11">
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="11"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="14"/>
-    </row>
-    <row r="41" spans="3:11">
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="11"/>
-      <c r="J41" s="14"/>
-      <c r="K41" s="14"/>
-    </row>
-    <row r="42" spans="3:11">
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="14"/>
-      <c r="K42" s="14"/>
-    </row>
-    <row r="43" spans="3:11">
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-    </row>
-    <row r="44" spans="3:11">
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="11"/>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
-    </row>
-    <row r="45" spans="3:11">
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="11"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
-    </row>
-    <row r="46" spans="3:11">
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-    </row>
-    <row r="47" spans="3:11">
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="14"/>
-      <c r="J47" s="14"/>
-      <c r="K47" s="14"/>
+    <row r="34" spans="7:9">
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13410,11 +14463,11 @@
       <c r="C9">
         <v>791.38082399999996</v>
       </c>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13" t="s">
+      <c r="N9" s="4"/>
+      <c r="O9" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="P9" s="13" t="s">
+      <c r="P9" s="4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -13425,13 +14478,13 @@
       <c r="C10">
         <v>695.81287599999996</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" t="s">
         <v>99</v>
       </c>
-      <c r="O10" s="11">
+      <c r="O10">
         <v>500.27759300000008</v>
       </c>
-      <c r="P10" s="11">
+      <c r="P10">
         <v>594.43553344444445</v>
       </c>
     </row>
@@ -13442,13 +14495,13 @@
       <c r="C11">
         <v>527.410031</v>
       </c>
-      <c r="N11" s="11" t="s">
+      <c r="N11" t="s">
         <v>100</v>
       </c>
-      <c r="O11" s="11">
+      <c r="O11">
         <v>5555.4812917667441</v>
       </c>
-      <c r="P11" s="11">
+      <c r="P11">
         <v>12447.904788325191</v>
       </c>
     </row>
@@ -13459,13 +14512,13 @@
       <c r="C12">
         <v>576.467668</v>
       </c>
-      <c r="N12" s="11" t="s">
+      <c r="N12" t="s">
         <v>101</v>
       </c>
-      <c r="O12" s="11">
+      <c r="O12">
         <v>10</v>
       </c>
-      <c r="P12" s="11">
+      <c r="P12">
         <v>9</v>
       </c>
     </row>
@@ -13473,76 +14526,69 @@
       <c r="B13">
         <v>495.25925899999999</v>
       </c>
-      <c r="N13" s="11" t="s">
+      <c r="N13" t="s">
         <v>111</v>
       </c>
-      <c r="O13" s="11">
+      <c r="O13">
         <v>8798.974701911895</v>
       </c>
-      <c r="P13" s="11"/>
     </row>
     <row r="14" spans="2:16">
-      <c r="N14" s="11" t="s">
+      <c r="N14" t="s">
         <v>102</v>
       </c>
-      <c r="O14" s="11">
+      <c r="O14">
         <v>0</v>
       </c>
-      <c r="P14" s="11"/>
     </row>
     <row r="15" spans="2:16">
-      <c r="N15" s="11" t="s">
+      <c r="N15" t="s">
         <v>103</v>
       </c>
-      <c r="O15" s="11">
+      <c r="O15">
         <v>17</v>
       </c>
-      <c r="P15" s="11"/>
     </row>
     <row r="16" spans="2:16">
-      <c r="N16" s="11" t="s">
+      <c r="N16" t="s">
         <v>104</v>
       </c>
-      <c r="O16" s="11">
+      <c r="O16">
         <v>-2.1846676115030039</v>
       </c>
-      <c r="P16" s="11"/>
     </row>
     <row r="17" spans="14:16">
-      <c r="N17" s="11" t="s">
+      <c r="N17" t="s">
         <v>105</v>
       </c>
-      <c r="O17" s="11">
+      <c r="O17">
         <v>2.1603458578222112E-2</v>
       </c>
-      <c r="P17" s="11"/>
     </row>
     <row r="18" spans="14:16">
-      <c r="N18" s="11" t="s">
+      <c r="N18" t="s">
         <v>106</v>
       </c>
-      <c r="O18" s="11">
+      <c r="O18">
         <v>1.7396067260750732</v>
       </c>
-      <c r="P18" s="11"/>
     </row>
     <row r="19" spans="14:16">
-      <c r="N19" s="16" t="s">
+      <c r="N19" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="O19" s="16">
-        <v>4.3206917156444223E-2</v>
-      </c>
-      <c r="P19" s="11"/>
+      <c r="O19" s="11">
+        <v>4.3206917156444202E-2</v>
+      </c>
     </row>
     <row r="20" spans="14:16" ht="15" thickBot="1">
-      <c r="N20" s="12" t="s">
+      <c r="N20" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="O20" s="12">
+      <c r="O20" s="3">
         <v>2.109815577833317</v>
       </c>
-      <c r="P20" s="12"/>
+      <c r="P20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
work on visualising the synced blinks per time bin; now also scaled per minute
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380B2009-E563-432D-9C2E-3F49BF5D4D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197B3E18-4A28-4CA0-BE08-90E6286451B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="603" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,10 +21,6 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">BlinkRateMinute!$F$2:$F$11</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">BlinkRateMinute!$P$2:$P$10</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">Sheet3!$B$3</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">Sheet3!$B$4:$B$13</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">Sheet3!$C$3</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">Sheet3!$C$4:$C$13</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$D$3</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$D$4:$D$13</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$E$3</definedName>
@@ -4238,36 +4234,6 @@
                   <c:y val="-7.8691147588244831E-2"/>
                 </c:manualLayout>
               </c:layout>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr>
-                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                        <a:solidFill>
-                          <a:schemeClr val="tx1">
-                            <a:lumMod val="65000"/>
-                            <a:lumOff val="35000"/>
-                          </a:schemeClr>
-                        </a:solidFill>
-                        <a:latin typeface="+mn-lt"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:defRPr>
-                    </a:pPr>
-                    <a:r>
-                      <a:rPr lang="en-US"/>
-                      <a:t>r=0.036</a:t>
-                    </a:r>
-                    <a:r>
-                      <a:rPr lang="en-US" baseline="0"/>
-                      <a:t>  p=.28</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -4735,6 +4701,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{4DFF839D-C16C-4082-A573-2E00517ECB81}">
           <cx:tx>
             <cx:txData>
+              <cx:f/>
               <cx:v>Dyads BPM</cx:v>
             </cx:txData>
           </cx:tx>
@@ -4750,6 +4717,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-722A-435E-990A-4B385DA554D8}">
           <cx:tx>
             <cx:txData>
+              <cx:f/>
               <cx:v>Triads BPM</cx:v>
             </cx:txData>
           </cx:tx>
@@ -11508,8 +11476,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="12819530" y="11679518"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="12794504" y="11507321"/>
+              <a:ext cx="4552202" cy="2705473"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -14404,6 +14372,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFC0AEBE-0304-40C9-AD55-B102AE5944DF}">
   <dimension ref="B3:P20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="14" max="14" width="14.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="2:16">
       <c r="B3" t="s">

</xml_diff>

<commit_message>
added the p values to the boxplots and added the additional data (5 triads, 1 dyad still missing- to be added)
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197B3E18-4A28-4CA0-BE08-90E6286451B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7446CE-58BC-4A6E-A13D-C97EEBB1F5B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="165">
   <si>
     <t>Group</t>
   </si>
@@ -482,25 +482,70 @@
     <t>Triad</t>
   </si>
   <si>
-    <t>2024 05 07 - triad S1 G2</t>
-  </si>
-  <si>
-    <t>2024 05 07 - triad S1 G4</t>
-  </si>
-  <si>
-    <t>TRIAD_2024_11_04_Seminar_Mun_Session_1_Group_1</t>
-  </si>
-  <si>
-    <t>DYAD_2024_11_04_Seminar_Mun_Session_1_Group_2</t>
-  </si>
-  <si>
-    <t>TRIAD_2024_11_11_Seminar_Mun_Session_1_Group_1</t>
-  </si>
-  <si>
-    <t>TRIAD_2024_11_18_Seminar_Mun_Session_1_Group_1</t>
-  </si>
-  <si>
     <t>Triads</t>
+  </si>
+  <si>
+    <t>not synced, confirmed by laura</t>
+  </si>
+  <si>
+    <t>synced, confirmed by laura</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> start: 2024-05-07 11:36:51.956</t>
+  </si>
+  <si>
+    <t>start: 2024-05-07 11:36:41.619</t>
+  </si>
+  <si>
+    <t>end: 2024-05-07 11:40:34.824</t>
+  </si>
+  <si>
+    <t>end: 2024-05-07 11:43:38.342</t>
+  </si>
+  <si>
+    <t>s: 2024-11-04 15:46:54.168</t>
+  </si>
+  <si>
+    <t>e: 2024-11-04 15:56:38.717</t>
+  </si>
+  <si>
+    <t>e:2024-11-04 17:15:10.815</t>
+  </si>
+  <si>
+    <t>s: 2024-11-04 17:06:11.026</t>
+  </si>
+  <si>
+    <t>s: 2024-11-11 15:49:25.519</t>
+  </si>
+  <si>
+    <t>e: 2024-11-11 15:57:00.444</t>
+  </si>
+  <si>
+    <t>s: 2024-11-18 15:50:30.315</t>
+  </si>
+  <si>
+    <t>e: 2024-11-18 16:00:45.857</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_05_07_Seminar_Wue_Session_1_Group_4_TS</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_05_07_Seminar_Wue_Session_1_Group_2_TS</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_11_04_Seminar_Mun_Session_1_Group_1_TS</t>
+  </si>
+  <si>
+    <t>DYAD_2024_11_04_Seminar_Mun_Session_1_Group_2_TS</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_11_11_Seminar_Mun_Session_1_Group_1_TS</t>
+  </si>
+  <si>
+    <t>TRIAD_2024_11_18_Seminar_Mun_Session_1_Group_1_TS</t>
+  </si>
+  <si>
+    <t>no file yet</t>
   </si>
 </sst>
 </file>
@@ -595,7 +640,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -618,6 +663,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12241,8 +12287,8 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="54.54296875" customWidth="1"/>
-    <col min="2" max="2" width="22.81640625" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="2" max="2" width="27.08984375" customWidth="1"/>
+    <col min="3" max="3" width="27.6328125" customWidth="1"/>
     <col min="4" max="4" width="10.81640625" customWidth="1"/>
     <col min="5" max="5" width="11.54296875" customWidth="1"/>
   </cols>
@@ -12363,6 +12409,9 @@
       <c r="E6">
         <v>0</v>
       </c>
+      <c r="F6" t="s">
+        <v>144</v>
+      </c>
       <c r="G6" t="s">
         <v>16</v>
       </c>
@@ -12502,7 +12551,7 @@
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" t="s">
+      <c r="A14" s="6" t="s">
         <v>68</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -12517,12 +12566,15 @@
       <c r="E14">
         <v>0</v>
       </c>
+      <c r="F14" t="s">
+        <v>145</v>
+      </c>
       <c r="G14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" t="s">
+      <c r="A15" s="6" t="s">
         <v>69</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -12536,6 +12588,9 @@
       </c>
       <c r="E15">
         <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>145</v>
       </c>
       <c r="G15" t="s">
         <v>37</v>
@@ -12698,38 +12753,78 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
-      <c r="A31" t="s">
-        <v>143</v>
-      </c>
-    </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>144</v>
+        <v>158</v>
+      </c>
+      <c r="B32" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" t="s">
+        <v>148</v>
       </c>
     </row>
-    <row r="36" spans="1:1">
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>159</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="C33" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>145</v>
+        <v>160</v>
+      </c>
+      <c r="B36" t="s">
+        <v>150</v>
+      </c>
+      <c r="C36" t="s">
+        <v>151</v>
       </c>
     </row>
-    <row r="37" spans="1:1">
-      <c r="A37" t="s">
-        <v>146</v>
+    <row r="37" spans="1:6">
+      <c r="A37" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>164</v>
       </c>
     </row>
-    <row r="38" spans="1:1">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>147</v>
+        <v>162</v>
+      </c>
+      <c r="B38" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38" t="s">
+        <v>155</v>
       </c>
     </row>
-    <row r="39" spans="1:1">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>148</v>
+        <v>163</v>
+      </c>
+      <c r="B39" t="s">
+        <v>156</v>
+      </c>
+      <c r="C39" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -14381,7 +14476,7 @@
         <v>91</v>
       </c>
       <c r="C3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="2:16">

</xml_diff>

<commit_message>
added the last dyad data; now the dataset is complete
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7446CE-58BC-4A6E-A13D-C97EEBB1F5B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5549F97B-5912-45E0-AA3D-F1168B50ACB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="28800" windowHeight="15370" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="164">
   <si>
     <t>Group</t>
   </si>
@@ -543,9 +543,6 @@
   </si>
   <si>
     <t>TRIAD_2024_11_18_Seminar_Mun_Session_1_Group_1_TS</t>
-  </si>
-  <si>
-    <t>no file yet</t>
   </si>
 </sst>
 </file>
@@ -640,7 +637,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -664,6 +661,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12787,18 +12785,16 @@
       </c>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>164</v>
-      </c>
+      <c r="F37" s="6"/>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">

</xml_diff>

<commit_message>
added come code to get the valid duration of each group conversation
</commit_message>
<xml_diff>
--- a/data/groups_info.xlsx
+++ b/data/groups_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BA6E67-AEA5-4B9D-9B95-AE7AF953F745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{410EE69A-719F-45BC-A52F-9D68984608CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="603" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15915" yWindow="0" windowWidth="12990" windowHeight="15585" tabRatio="279" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="SyncedBlink%" sheetId="3" r:id="rId4"/>
     <sheet name="MeanBlinkAsyncMS" sheetId="4" r:id="rId5"/>
     <sheet name="AsyncBlinkTimeWindow" sheetId="6" r:id="rId6"/>
+    <sheet name="Discussion" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">BlinkDurationMS!$F$2:$F$12</definedName>
@@ -55,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="235">
   <si>
     <t>Group</t>
   </si>
@@ -658,6 +659,134 @@
   </si>
   <si>
     <t>triads [0 : 250ms]</t>
+  </si>
+  <si>
+    <t>Blink Duration</t>
+  </si>
+  <si>
+    <t>Blink Rate</t>
+  </si>
+  <si>
+    <t>% synced blinks</t>
+  </si>
+  <si>
+    <t>Asynced blinks temporal</t>
+  </si>
+  <si>
+    <t>Mean Asynced blinks time</t>
+  </si>
+  <si>
+    <t>no significant diff</t>
+  </si>
+  <si>
+    <t>higher per dyads</t>
+  </si>
+  <si>
+    <t>higher mean async for triads</t>
+  </si>
+  <si>
+    <t>no sig diff between dyads and tryads;</t>
+  </si>
+  <si>
+    <t>ÇAKIR&amp;HUCKAUF 2024</t>
+  </si>
+  <si>
+    <t>less in self-mirror than in dyad-mirror</t>
+  </si>
+  <si>
+    <t>Studies</t>
+  </si>
+  <si>
+    <t>ours</t>
+  </si>
+  <si>
+    <t>more sig bins in dyads, different distribution</t>
+  </si>
+  <si>
+    <t>no significant difference</t>
+  </si>
+  <si>
+    <t>higher in dyad than in self-mirror</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no significant difference; </t>
+  </si>
+  <si>
+    <t>Ours - explanations</t>
+  </si>
+  <si>
+    <t>C&amp;H 2024 - exaplanations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The blink rate is within the normal standard values for conversations (26.1[1]-for one person talking in a dyad, 26[2]-for one person talking without recalling info). This value is lower for triads, however this can be explained by the presence of a bystander within the group during the conversation who would behave as in a 'lecture' [1]. (But check lit on blink rate in triads) ([1]Al-Abdulmunem&amp;Briggs, 1999; [2]Bentivoglio et al. 2004);
+The Absolute amount of blinks could be regarded as a factor responsible for the observed effects (on the mean async blinks time). In short, the 'blink rate' difference could affect the 'mean asynced blinks time'.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Even though there is no significant difference between dyads and triads, we can see a higher avg for dyads (0.61) compared to triads (0.51). The non-significant difference seen in the blink rate could have affected the difference in the % synced blinks, however, a follow up study with a bigger population is needed to confirm this idea. </t>
+  </si>
+  <si>
+    <t>During the same task, the temporal structure of the asynced blinks was very similar, with the only slight perceivable difference not significant (see timewidow [0-250ms]).
+Although the blink rate was higher in the dyad setting and for triads there was a higher lag  between the onset reference blink and test blink, these did not affect the general temporal structure seen for dyads and triads.
+This scructure is similar to previous literature on dyadic interaction [ref C&amp;H2024]</t>
+  </si>
+  <si>
+    <r>
+      <t>The higher mean asynced blinks time f</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">r triads (lag between the reference blink onset and the synced blink onset of the other participant) could be an effect of the significantly lower blink rate in triads compared to dyads. </t>
+    </r>
+  </si>
+  <si>
+    <t>Currently using for Gaze analysis</t>
+  </si>
+  <si>
+    <t>Potential using for Gaze analysis</t>
+  </si>
+  <si>
+    <t>5 dyads - 3234s</t>
+  </si>
+  <si>
+    <t>6 triads - 3031s</t>
+  </si>
+  <si>
+    <t>6 dyads -&gt; +1</t>
+  </si>
+  <si>
+    <t>11-12 triads -&gt; +5,6</t>
+  </si>
+  <si>
+    <t>dyad - triad</t>
+  </si>
+  <si>
+    <t>VR - free flow conv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VR - don't see the gaze: blink; </t>
+  </si>
+  <si>
+    <t>don't look at eachother; &lt; add to these</t>
+  </si>
+  <si>
+    <t>similar setting in non-vr</t>
   </si>
 </sst>
 </file>
@@ -773,7 +902,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -800,27 +929,47 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="22">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -6430,12 +6579,6 @@
     <cx:plotArea>
       <cx:plotAreaRegion>
         <cx:series layoutId="boxWhisker" uniqueId="{8E42B4CF-C767-4F7B-8021-4E2E2439F66F}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f/>
-              <cx:v>Dyads</cx:v>
-            </cx:txData>
-          </cx:tx>
           <cx:spPr>
             <a:noFill/>
           </cx:spPr>
@@ -6446,12 +6589,6 @@
           </cx:layoutPr>
         </cx:series>
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-4CC7-4FA6-8D6A-38409316E009}">
-          <cx:tx>
-            <cx:txData>
-              <cx:f/>
-              <cx:v>Triads</cx:v>
-            </cx:txData>
-          </cx:tx>
           <cx:spPr>
             <a:noFill/>
           </cx:spPr>
@@ -15260,8 +15397,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="13141325" y="3079750"/>
-              <a:ext cx="4025900" cy="2841625"/>
+              <a:off x="13674725" y="2978150"/>
+              <a:ext cx="4124325" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -15641,8 +15778,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="12384929" y="11862921"/>
-              <a:ext cx="4441077" cy="2788023"/>
+              <a:off x="12794504" y="11462871"/>
+              <a:ext cx="4552202" cy="2699123"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -15965,8 +16102,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="7748588" y="5499100"/>
-              <a:ext cx="3211512" cy="2355851"/>
+              <a:off x="7856538" y="5314950"/>
+              <a:ext cx="3322637" cy="2270126"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -16048,8 +16185,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="164773" y="3071868"/>
-              <a:ext cx="4057758" cy="3383565"/>
+              <a:off x="164773" y="2970268"/>
+              <a:ext cx="4057758" cy="3266090"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -16247,6 +16384,21 @@
 </table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AE3128D6-0977-4CDB-9564-6576F6CC0F00}" name="Table12" displayName="Table12" ref="B3:G9" totalsRowShown="0" headerRowDxfId="7" dataDxfId="1">
+  <autoFilter ref="B3:G9" xr:uid="{AE3128D6-0977-4CDB-9564-6576F6CC0F00}"/>
+  <tableColumns count="6">
+    <tableColumn id="7" xr3:uid="{9ADAD039-B1E9-4CE9-A97A-F011BE916F7E}" name="Studies" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{82438DF6-BD05-4592-A8DD-7774EC290540}" name="Blink Duration" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{73A7EFA3-1D5A-46CB-8FDD-FC9B98AFF790}" name="Blink Rate" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{870B7377-D9C2-43BC-BF44-555251957991}" name="% synced blinks" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{2CBBC7E0-C34D-4EDC-BAF8-1044465DAD77}" name="Mean Asynced blinks time" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{0FE01176-586C-4503-854F-0ADC1D5FE9ED}" name="Asynced blinks temporal" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FED66298-7890-498B-98F2-11D90C33227F}" name="Table8" displayName="Table8" ref="I1:N15" totalsRowShown="0">
   <autoFilter ref="I1:N15" xr:uid="{FED66298-7890-498B-98F2-11D90C33227F}"/>
@@ -16263,13 +16415,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AD080257-BFA1-460B-B07A-36A64761A16A}" name="Table1" displayName="Table1" ref="C1:F12" totalsRowShown="0" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AD080257-BFA1-460B-B07A-36A64761A16A}" name="Table1" displayName="Table1" ref="C1:F12" totalsRowShown="0" dataDxfId="21">
   <autoFilter ref="C1:F12" xr:uid="{AD080257-BFA1-460B-B07A-36A64761A16A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{4F27821A-74B4-4054-BD57-59CB04F69638}" name="Group" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{40FF8A35-FADD-40F8-9C7C-8272D131492D}" name="P1" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{57E54AEA-9EE5-4960-BBF2-37C5CACE9F4B}" name="P2" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{9B5C91BC-FC38-40B1-900E-1D679A89BBE9}" name="P1_P2_AVG" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{4F27821A-74B4-4054-BD57-59CB04F69638}" name="Group" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{40FF8A35-FADD-40F8-9C7C-8272D131492D}" name="P1" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{57E54AEA-9EE5-4960-BBF2-37C5CACE9F4B}" name="P2" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{9B5C91BC-FC38-40B1-900E-1D679A89BBE9}" name="P1_P2_AVG" dataDxfId="17">
       <calculatedColumnFormula>AVERAGE(Table1[[#This Row],[P1]]:Table1[[#This Row],[P2]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -16278,23 +16430,23 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1613B083-0BCB-449A-A18A-943282863FFE}" name="Table2" displayName="Table2" ref="I1:P15" totalsRowShown="0" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1613B083-0BCB-449A-A18A-943282863FFE}" name="Table2" displayName="Table2" ref="I1:P15" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="I1:P15" xr:uid="{1613B083-0BCB-449A-A18A-943282863FFE}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{4B00F100-EEAB-4176-8F7C-64576AF95E9C}" name="Group" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{0C1C6D39-9F0B-4EFB-8FFF-6819FFEE1A73}" name="P1" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{4B646295-E6BA-4208-9890-BF77B7CC4DB0}" name="P2" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{90141FC2-ED7D-4A6B-AFC1-04A51D13EAB7}" name="P3" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{45EA91F4-80A5-4D09-8BA5-58CA8E684F50}" name="avg_P1P2" dataDxfId="3">
+    <tableColumn id="1" xr3:uid="{4B00F100-EEAB-4176-8F7C-64576AF95E9C}" name="Group" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{0C1C6D39-9F0B-4EFB-8FFF-6819FFEE1A73}" name="P1" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{4B646295-E6BA-4208-9890-BF77B7CC4DB0}" name="P2" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{90141FC2-ED7D-4A6B-AFC1-04A51D13EAB7}" name="P3" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{45EA91F4-80A5-4D09-8BA5-58CA8E684F50}" name="avg_P1P2" dataDxfId="11">
       <calculatedColumnFormula>AVERAGE(Table2[[#This Row],[P1]:[P2]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8D95483F-1D1F-4BC0-9A13-DB0617692381}" name="avg_P1P3" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{8D95483F-1D1F-4BC0-9A13-DB0617692381}" name="avg_P1P3" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(J2,L2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{CEE85F33-BF2F-4114-920C-22ACF0374CF1}" name="avg_P2P3" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{CEE85F33-BF2F-4114-920C-22ACF0374CF1}" name="avg_P2P3" dataDxfId="9">
       <calculatedColumnFormula>AVERAGE(Table2[[#This Row],[P2]]:Table2[[#This Row],[P3]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{2974D60E-6187-4B53-9C0A-D6CCD473C533}" name="avg_P123" dataDxfId="0">
+    <tableColumn id="8" xr3:uid="{2974D60E-6187-4B53-9C0A-D6CCD473C533}" name="avg_P123" dataDxfId="8">
       <calculatedColumnFormula>AVERAGE(Table2[[#This Row],[P1]],Table2[[#This Row],[P2]],Table2[[#This Row],[P3]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -16641,14 +16793,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.5703125" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="54.54296875" customWidth="1"/>
+    <col min="2" max="2" width="27.1796875" customWidth="1"/>
+    <col min="3" max="3" width="27.54296875" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -17176,6 +17328,30 @@
       </c>
       <c r="C39" t="s">
         <v>153</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="B42" t="s">
+        <v>224</v>
+      </c>
+      <c r="C42" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="B43" t="s">
+        <v>226</v>
+      </c>
+      <c r="C43" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="B44" t="s">
+        <v>227</v>
+      </c>
+      <c r="C44" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -17187,19 +17363,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3C3795-97EB-4298-A25F-860B0A0E50BA}">
   <dimension ref="B1:N44"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.26953125" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
     <col min="3" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" customWidth="1"/>
-    <col min="13" max="13" width="27.140625" customWidth="1"/>
-    <col min="14" max="14" width="30.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
+    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="10" max="10" width="11.81640625" customWidth="1"/>
+    <col min="11" max="11" width="14.26953125" customWidth="1"/>
+    <col min="12" max="12" width="9.7265625" customWidth="1"/>
+    <col min="13" max="13" width="27.1796875" customWidth="1"/>
+    <col min="14" max="14" width="30.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14">
@@ -17748,7 +17924,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="27" spans="3:12" ht="15.75" thickBot="1"/>
+    <row r="27" spans="3:12" ht="15" thickBot="1"/>
     <row r="28" spans="3:12">
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
@@ -17870,7 +18046,7 @@
         <v>1.4291769235957907</v>
       </c>
     </row>
-    <row r="35" spans="2:12" ht="15.75" thickBot="1">
+    <row r="35" spans="2:12" ht="15" thickBot="1">
       <c r="D35" s="3" t="s">
         <v>162</v>
       </c>
@@ -17901,7 +18077,7 @@
         <v>0.17488621060546347</v>
       </c>
     </row>
-    <row r="38" spans="2:12" ht="15.75" thickBot="1">
+    <row r="38" spans="2:12" ht="15" thickBot="1">
       <c r="J38" s="3" t="s">
         <v>108</v>
       </c>
@@ -17930,13 +18106,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08CBB891-F584-4F5A-A553-41469C7D6F94}">
   <dimension ref="C1:AO167"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="57.140625" customWidth="1"/>
+    <col min="3" max="3" width="57.1796875" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="9" max="9" width="58.28515625" customWidth="1"/>
+    <col min="9" max="9" width="58.26953125" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="15" width="11.85546875" customWidth="1"/>
+    <col min="14" max="15" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:16">
@@ -18573,7 +18749,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="48" spans="4:23" ht="15.75" thickBot="1">
+    <row r="48" spans="4:23" ht="15" thickBot="1">
       <c r="D48">
         <v>2.4711409999999998</v>
       </c>
@@ -18741,7 +18917,7 @@
       <c r="V59" s="9"/>
       <c r="W59" s="9"/>
     </row>
-    <row r="60" spans="4:23" ht="15.75" thickBot="1">
+    <row r="60" spans="4:23" ht="15" thickBot="1">
       <c r="K60" s="3" t="s">
         <v>108</v>
       </c>
@@ -18867,7 +19043,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="77" spans="4:6" ht="15.75" thickBot="1"/>
+    <row r="77" spans="4:6" ht="15" thickBot="1"/>
     <row r="78" spans="4:6">
       <c r="D78" s="8" t="s">
         <v>116</v>
@@ -18909,7 +19085,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="83" spans="4:17" ht="15.75" thickBot="1">
+    <row r="83" spans="4:17" ht="15" thickBot="1">
       <c r="D83" s="3" t="s">
         <v>101</v>
       </c>
@@ -18926,7 +19102,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="85" spans="4:17" ht="15.75" thickBot="1">
+    <row r="85" spans="4:17" ht="15" thickBot="1">
       <c r="D85" t="s">
         <v>121</v>
       </c>
@@ -19019,7 +19195,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="89" spans="4:17" ht="15.75" thickBot="1">
+    <row r="89" spans="4:17" ht="15" thickBot="1">
       <c r="D89" s="3" t="s">
         <v>124</v>
       </c>
@@ -19039,7 +19215,7 @@
         <v>2.1493368459329587</v>
       </c>
     </row>
-    <row r="90" spans="4:17" ht="15.75" thickBot="1">
+    <row r="90" spans="4:17" ht="15" thickBot="1">
       <c r="O90" t="s">
         <v>161</v>
       </c>
@@ -19047,7 +19223,7 @@
         <v>9.843683670970256E-2</v>
       </c>
     </row>
-    <row r="91" spans="4:17" ht="15.75" thickBot="1">
+    <row r="91" spans="4:17" ht="15" thickBot="1">
       <c r="D91" s="4"/>
       <c r="E91" s="4" t="s">
         <v>130</v>
@@ -19110,7 +19286,7 @@
         <v>37.855258279391578</v>
       </c>
     </row>
-    <row r="93" spans="4:17" ht="15.75" thickBot="1">
+    <row r="93" spans="4:17" ht="15" thickBot="1">
       <c r="D93" s="3" t="s">
         <v>136</v>
       </c>
@@ -19144,125 +19320,123 @@
         <v>115</v>
       </c>
     </row>
-    <row r="98" spans="4:35" ht="15.75" thickBot="1"/>
+    <row r="98" spans="4:35" ht="15" thickBot="1"/>
     <row r="99" spans="4:35">
-      <c r="D99" s="17" t="s">
+      <c r="D99" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="E99" s="17"/>
+      <c r="E99" s="8"/>
     </row>
     <row r="100" spans="4:35">
-      <c r="D100" s="14" t="s">
+      <c r="D100" t="s">
         <v>117</v>
       </c>
-      <c r="E100" s="14">
+      <c r="E100">
         <v>0.36556131816160797</v>
       </c>
     </row>
     <row r="101" spans="4:35">
-      <c r="D101" s="14" t="s">
+      <c r="D101" t="s">
         <v>118</v>
       </c>
-      <c r="E101" s="14">
+      <c r="E101">
         <v>0.13363507733605237</v>
       </c>
     </row>
     <row r="102" spans="4:35">
-      <c r="D102" s="14" t="s">
+      <c r="D102" t="s">
         <v>119</v>
       </c>
-      <c r="E102" s="14">
+      <c r="E102">
         <v>3.7372308151169306E-2</v>
       </c>
     </row>
     <row r="103" spans="4:35">
-      <c r="D103" s="14" t="s">
+      <c r="D103" t="s">
         <v>120</v>
       </c>
-      <c r="E103" s="14">
+      <c r="E103">
         <v>10.910273656348574</v>
       </c>
     </row>
-    <row r="104" spans="4:35" ht="15.75" thickBot="1">
-      <c r="D104" s="15" t="s">
+    <row r="104" spans="4:35" ht="15" thickBot="1">
+      <c r="D104" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="E104" s="15">
+      <c r="E104" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="4:35" ht="15.75" thickBot="1">
+    <row r="106" spans="4:35" ht="15" thickBot="1">
       <c r="D106" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="107" spans="4:35">
-      <c r="D107" s="16"/>
-      <c r="E107" s="16" t="s">
+      <c r="D107" s="4"/>
+      <c r="E107" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F107" s="16" t="s">
+      <c r="F107" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="G107" s="16" t="s">
+      <c r="G107" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="H107" s="16" t="s">
+      <c r="H107" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="I107" s="16" t="s">
+      <c r="I107" s="4" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="108" spans="4:35">
-      <c r="D108" s="14" t="s">
+      <c r="D108" t="s">
         <v>122</v>
       </c>
-      <c r="E108" s="14">
+      <c r="E108">
         <v>1</v>
       </c>
-      <c r="F108" s="14">
+      <c r="F108">
         <v>165.24693246071752</v>
       </c>
-      <c r="G108" s="14">
+      <c r="G108">
         <v>165.24693246071752</v>
       </c>
-      <c r="H108" s="14">
+      <c r="H108">
         <v>1.3882322155037088</v>
       </c>
-      <c r="I108" s="14">
+      <c r="I108">
         <v>0.26891717148188249</v>
       </c>
     </row>
     <row r="109" spans="4:35">
-      <c r="D109" s="14" t="s">
+      <c r="D109" t="s">
         <v>123</v>
       </c>
-      <c r="E109" s="14">
+      <c r="E109">
         <v>9</v>
       </c>
-      <c r="F109" s="14">
+      <c r="F109">
         <v>1071.3066413077231</v>
       </c>
-      <c r="G109" s="14">
+      <c r="G109">
         <v>119.03407125641368</v>
       </c>
-      <c r="H109" s="14"/>
-      <c r="I109" s="14"/>
-    </row>
-    <row r="110" spans="4:35" ht="15.75" thickBot="1">
-      <c r="D110" s="15" t="s">
+    </row>
+    <row r="110" spans="4:35" ht="15" thickBot="1">
+      <c r="D110" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E110" s="15">
+      <c r="E110" s="3">
         <v>10</v>
       </c>
-      <c r="F110" s="15">
+      <c r="F110" s="3">
         <v>1236.5535737684406</v>
       </c>
-      <c r="G110" s="15"/>
-      <c r="H110" s="15"/>
-      <c r="I110" s="15"/>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
+      <c r="I110" s="3"/>
       <c r="AG110" t="s">
         <v>115</v>
       </c>
@@ -19270,133 +19444,133 @@
         <v>198</v>
       </c>
     </row>
-    <row r="111" spans="4:35" ht="15.75" thickBot="1"/>
+    <row r="111" spans="4:35" ht="15" thickBot="1"/>
     <row r="112" spans="4:35">
-      <c r="D112" s="16"/>
-      <c r="E112" s="16" t="s">
+      <c r="D112" s="4"/>
+      <c r="E112" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F112" s="16" t="s">
+      <c r="F112" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G112" s="16" t="s">
+      <c r="G112" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="H112" s="16" t="s">
+      <c r="H112" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="I112" s="16" t="s">
+      <c r="I112" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="J112" s="16" t="s">
+      <c r="J112" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="K112" s="16" t="s">
+      <c r="K112" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="L112" s="16" t="s">
+      <c r="L112" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="AG112" s="17" t="s">
+      <c r="AG112" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="AH112" s="17"/>
+      <c r="AH112" s="8"/>
     </row>
     <row r="113" spans="4:41">
-      <c r="D113" s="14" t="s">
+      <c r="D113" t="s">
         <v>125</v>
       </c>
-      <c r="E113" s="14">
+      <c r="E113">
         <v>6.1046276707605944</v>
       </c>
-      <c r="F113" s="14">
+      <c r="F113">
         <v>13.419269180023679</v>
       </c>
-      <c r="G113" s="14">
+      <c r="G113">
         <v>0.45491506198028453</v>
       </c>
-      <c r="H113" s="14">
+      <c r="H113">
         <v>0.65994487461269657</v>
       </c>
-      <c r="I113" s="14">
+      <c r="I113">
         <v>-24.25186822434717</v>
       </c>
-      <c r="J113" s="14">
+      <c r="J113">
         <v>36.461123565868363</v>
       </c>
-      <c r="K113" s="14">
+      <c r="K113">
         <v>-24.25186822434717</v>
       </c>
-      <c r="L113" s="14">
+      <c r="L113">
         <v>36.461123565868363</v>
       </c>
-      <c r="AG113" s="14" t="s">
+      <c r="AG113" t="s">
         <v>117</v>
       </c>
-      <c r="AH113" s="14">
+      <c r="AH113">
         <v>0.55522926444419129</v>
       </c>
     </row>
-    <row r="114" spans="4:41" ht="15.75" thickBot="1">
-      <c r="D114" s="15" t="s">
+    <row r="114" spans="4:41" ht="15" thickBot="1">
+      <c r="D114" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E114" s="15">
+      <c r="E114" s="3">
         <v>0.42641624042422033</v>
       </c>
-      <c r="F114" s="15">
+      <c r="F114" s="3">
         <v>0.36191174518166136</v>
       </c>
-      <c r="G114" s="15">
+      <c r="G114" s="3">
         <v>1.1782326661163787</v>
       </c>
-      <c r="H114" s="15">
+      <c r="H114" s="3">
         <v>0.26891717148188271</v>
       </c>
-      <c r="I114" s="15">
+      <c r="I114" s="3">
         <v>-0.39228500623927376</v>
       </c>
-      <c r="J114" s="15">
+      <c r="J114" s="3">
         <v>1.2451174870877144</v>
       </c>
-      <c r="K114" s="15">
+      <c r="K114" s="3">
         <v>-0.39228500623927376</v>
       </c>
-      <c r="L114" s="15">
+      <c r="L114" s="3">
         <v>1.2451174870877144</v>
       </c>
-      <c r="AG114" s="14" t="s">
+      <c r="AG114" t="s">
         <v>118</v>
       </c>
-      <c r="AH114" s="14">
+      <c r="AH114">
         <v>0.30827953609523767</v>
       </c>
     </row>
     <row r="115" spans="4:41">
-      <c r="AG115" s="14" t="s">
+      <c r="AG115" t="s">
         <v>119</v>
       </c>
-      <c r="AH115" s="14">
+      <c r="AH115">
         <v>0.25063616410317419</v>
       </c>
     </row>
     <row r="116" spans="4:41">
-      <c r="AG116" s="14" t="s">
+      <c r="AG116" t="s">
         <v>120</v>
       </c>
-      <c r="AH116" s="14">
+      <c r="AH116">
         <v>4.505428874124374</v>
       </c>
     </row>
-    <row r="117" spans="4:41" ht="15.75" thickBot="1">
-      <c r="AG117" s="15" t="s">
+    <row r="117" spans="4:41" ht="15" thickBot="1">
+      <c r="AG117" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="AH117" s="15">
+      <c r="AH117" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="119" spans="4:41" ht="15.75" thickBot="1">
+    <row r="119" spans="4:41" ht="15" thickBot="1">
       <c r="T119" s="6" t="s">
         <v>88</v>
       </c>
@@ -19420,20 +19594,20 @@
       <c r="V120">
         <v>36.113652999999999</v>
       </c>
-      <c r="AG120" s="16"/>
-      <c r="AH120" s="16" t="s">
+      <c r="AG120" s="4"/>
+      <c r="AH120" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="AI120" s="16" t="s">
+      <c r="AI120" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="AJ120" s="16" t="s">
+      <c r="AJ120" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="AK120" s="16" t="s">
+      <c r="AK120" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="AL120" s="20" t="s">
+      <c r="AL120" s="14" t="s">
         <v>129</v>
       </c>
     </row>
@@ -19447,22 +19621,22 @@
       <c r="V121">
         <v>29.803229999999999</v>
       </c>
-      <c r="AG121" s="14" t="s">
+      <c r="AG121" t="s">
         <v>122</v>
       </c>
-      <c r="AH121" s="14">
+      <c r="AH121">
         <v>1</v>
       </c>
-      <c r="AI121" s="14">
+      <c r="AI121">
         <v>108.55944009975204</v>
       </c>
-      <c r="AJ121" s="14">
+      <c r="AJ121">
         <v>108.55944009975204</v>
       </c>
-      <c r="AK121" s="14">
+      <c r="AK121">
         <v>5.3480482740961506</v>
       </c>
-      <c r="AL121" s="21">
+      <c r="AL121" s="6">
         <v>3.9291762492268782E-2</v>
       </c>
     </row>
@@ -19476,22 +19650,20 @@
       <c r="V122">
         <v>22.608398000000001</v>
       </c>
-      <c r="AG122" s="14" t="s">
+      <c r="AG122" t="s">
         <v>123</v>
       </c>
-      <c r="AH122" s="14">
+      <c r="AH122">
         <v>12</v>
       </c>
-      <c r="AI122" s="14">
+      <c r="AI122">
         <v>243.5866720775235</v>
       </c>
-      <c r="AJ122" s="14">
+      <c r="AJ122">
         <v>20.298889339793625</v>
       </c>
-      <c r="AK122" s="14"/>
-      <c r="AL122" s="14"/>
-    </row>
-    <row r="123" spans="4:41" ht="15.75" thickBot="1">
+    </row>
+    <row r="123" spans="4:41" ht="15" thickBot="1">
       <c r="T123">
         <v>7.7812380000000001</v>
       </c>
@@ -19501,20 +19673,20 @@
       <c r="V123">
         <v>58.124909000000002</v>
       </c>
-      <c r="AG123" s="15" t="s">
+      <c r="AG123" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="AH123" s="15">
+      <c r="AH123" s="3">
         <v>13</v>
       </c>
-      <c r="AI123" s="15">
+      <c r="AI123" s="3">
         <v>352.14611217727554</v>
       </c>
-      <c r="AJ123" s="15"/>
-      <c r="AK123" s="15"/>
-      <c r="AL123" s="15"/>
-    </row>
-    <row r="124" spans="4:41" ht="15.75" thickBot="1">
+      <c r="AJ123" s="3"/>
+      <c r="AK123" s="3"/>
+      <c r="AL123" s="3"/>
+    </row>
+    <row r="124" spans="4:41" ht="15" thickBot="1">
       <c r="T124">
         <v>8.8605520000000002</v>
       </c>
@@ -19535,29 +19707,29 @@
       <c r="V125">
         <v>10.206614999999999</v>
       </c>
-      <c r="AG125" s="16"/>
-      <c r="AH125" s="16" t="s">
+      <c r="AG125" s="4"/>
+      <c r="AH125" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="AI125" s="16" t="s">
+      <c r="AI125" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="AJ125" s="16" t="s">
+      <c r="AJ125" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="AK125" s="16" t="s">
+      <c r="AK125" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="AL125" s="16" t="s">
+      <c r="AL125" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="AM125" s="16" t="s">
+      <c r="AM125" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="AN125" s="16" t="s">
+      <c r="AN125" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="AO125" s="16" t="s">
+      <c r="AO125" s="4" t="s">
         <v>135</v>
       </c>
     </row>
@@ -19571,35 +19743,35 @@
       <c r="V126">
         <v>18.789473999999998</v>
       </c>
-      <c r="AG126" s="14" t="s">
+      <c r="AG126" t="s">
         <v>125</v>
       </c>
-      <c r="AH126" s="14">
+      <c r="AH126">
         <v>1.96225130828822</v>
       </c>
-      <c r="AI126" s="14">
+      <c r="AI126">
         <v>4.6027306111102844</v>
       </c>
-      <c r="AJ126" s="14">
+      <c r="AJ126">
         <v>0.42632330111861139</v>
       </c>
-      <c r="AK126" s="14">
+      <c r="AK126">
         <v>0.67741986300536028</v>
       </c>
-      <c r="AL126" s="14">
+      <c r="AL126">
         <v>-8.06623719870095</v>
       </c>
-      <c r="AM126" s="14">
+      <c r="AM126">
         <v>11.99073981527739</v>
       </c>
-      <c r="AN126" s="14">
+      <c r="AN126">
         <v>-8.06623719870095</v>
       </c>
-      <c r="AO126" s="14">
+      <c r="AO126">
         <v>11.99073981527739</v>
       </c>
     </row>
-    <row r="127" spans="4:41" ht="15.75" thickBot="1">
+    <row r="127" spans="4:41" ht="15" thickBot="1">
       <c r="T127">
         <v>13.606121</v>
       </c>
@@ -19610,31 +19782,31 @@
         <v>34.287424999999999</v>
       </c>
       <c r="X127" s="6"/>
-      <c r="AG127" s="15" t="s">
+      <c r="AG127" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="AH127" s="15">
+      <c r="AH127" s="3">
         <v>0.54636490428133633</v>
       </c>
-      <c r="AI127" s="15">
+      <c r="AI127" s="3">
         <v>0.23625724498144463</v>
       </c>
-      <c r="AJ127" s="15">
+      <c r="AJ127" s="3">
         <v>2.3125847604133671</v>
       </c>
-      <c r="AK127" s="15">
+      <c r="AK127" s="3">
         <v>3.9291762492268782E-2</v>
       </c>
-      <c r="AL127" s="15">
+      <c r="AL127" s="3">
         <v>3.1604587813931384E-2</v>
       </c>
-      <c r="AM127" s="15">
+      <c r="AM127" s="3">
         <v>1.0611252207487412</v>
       </c>
-      <c r="AN127" s="15">
+      <c r="AN127" s="3">
         <v>3.1604587813931384E-2</v>
       </c>
-      <c r="AO127" s="15">
+      <c r="AO127" s="3">
         <v>1.0611252207487412</v>
       </c>
     </row>
@@ -19674,7 +19846,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="131" spans="20:38" ht="15.75" thickBot="1">
+    <row r="131" spans="20:38" ht="15" thickBot="1">
       <c r="T131">
         <v>14.677982999999999</v>
       </c>
@@ -19695,10 +19867,10 @@
       <c r="V132">
         <v>28.883882</v>
       </c>
-      <c r="AG132" s="17" t="s">
+      <c r="AG132" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="AH132" s="17"/>
+      <c r="AH132" s="8"/>
     </row>
     <row r="133" spans="20:38">
       <c r="T133">
@@ -19710,201 +19882,199 @@
       <c r="V133">
         <v>28.657671000000001</v>
       </c>
-      <c r="AG133" s="14" t="s">
+      <c r="AG133" t="s">
         <v>117</v>
       </c>
-      <c r="AH133" s="14">
+      <c r="AH133">
         <v>0.12237744065125283</v>
       </c>
     </row>
     <row r="134" spans="20:38">
-      <c r="AG134" s="14" t="s">
+      <c r="AG134" t="s">
         <v>118</v>
       </c>
-      <c r="AH134" s="14">
+      <c r="AH134">
         <v>1.4976237980350908E-2</v>
       </c>
     </row>
     <row r="135" spans="20:38">
-      <c r="AG135" s="14" t="s">
+      <c r="AG135" t="s">
         <v>119</v>
       </c>
-      <c r="AH135" s="14">
+      <c r="AH135">
         <v>-6.7109075521286518E-2</v>
       </c>
     </row>
     <row r="136" spans="20:38">
-      <c r="AG136" s="14" t="s">
+      <c r="AG136" t="s">
         <v>120</v>
       </c>
-      <c r="AH136" s="14">
+      <c r="AH136">
         <v>5.3764322758177139</v>
       </c>
     </row>
-    <row r="137" spans="20:38" ht="15.75" thickBot="1">
-      <c r="AG137" s="15" t="s">
+    <row r="137" spans="20:38" ht="15" thickBot="1">
+      <c r="AG137" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="AH137" s="15">
+      <c r="AH137" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="139" spans="20:38" ht="15.75" thickBot="1">
+    <row r="139" spans="20:38" ht="15" thickBot="1">
       <c r="AG139" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="140" spans="20:38">
-      <c r="AG140" s="16"/>
-      <c r="AH140" s="16" t="s">
+      <c r="AG140" s="4"/>
+      <c r="AH140" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="AI140" s="16" t="s">
+      <c r="AI140" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="AJ140" s="16" t="s">
+      <c r="AJ140" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="AK140" s="16" t="s">
+      <c r="AK140" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="AL140" s="16" t="s">
+      <c r="AL140" s="4" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="141" spans="20:38">
-      <c r="AG141" s="14" t="s">
+      <c r="AG141" t="s">
         <v>122</v>
       </c>
-      <c r="AH141" s="14">
+      <c r="AH141">
         <v>1</v>
       </c>
-      <c r="AI141" s="14">
+      <c r="AI141">
         <v>5.2738239798222253</v>
       </c>
-      <c r="AJ141" s="14">
+      <c r="AJ141">
         <v>5.2738239798222253</v>
       </c>
-      <c r="AK141" s="14">
+      <c r="AK141">
         <v>0.1824472288828155</v>
       </c>
-      <c r="AL141" s="14">
+      <c r="AL141">
         <v>0.67684228954421721</v>
       </c>
     </row>
     <row r="142" spans="20:38">
-      <c r="AG142" s="14" t="s">
+      <c r="AG142" t="s">
         <v>123</v>
       </c>
-      <c r="AH142" s="14">
+      <c r="AH142">
         <v>12</v>
       </c>
-      <c r="AI142" s="14">
+      <c r="AI142">
         <v>346.87228819745332</v>
       </c>
-      <c r="AJ142" s="14">
+      <c r="AJ142">
         <v>28.906024016454442</v>
       </c>
-      <c r="AK142" s="14"/>
-      <c r="AL142" s="14"/>
-    </row>
-    <row r="143" spans="20:38" ht="15.75" thickBot="1">
-      <c r="AG143" s="15" t="s">
+    </row>
+    <row r="143" spans="20:38" ht="15" thickBot="1">
+      <c r="AG143" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="AH143" s="15">
+      <c r="AH143" s="3">
         <v>13</v>
       </c>
-      <c r="AI143" s="15">
+      <c r="AI143" s="3">
         <v>352.14611217727554</v>
       </c>
-      <c r="AJ143" s="15"/>
-      <c r="AK143" s="15"/>
-      <c r="AL143" s="15"/>
-    </row>
-    <row r="144" spans="20:38" ht="15.75" thickBot="1"/>
+      <c r="AJ143" s="3"/>
+      <c r="AK143" s="3"/>
+      <c r="AL143" s="3"/>
+    </row>
+    <row r="144" spans="20:38" ht="15" thickBot="1"/>
     <row r="145" spans="33:41">
-      <c r="AG145" s="16"/>
-      <c r="AH145" s="16" t="s">
+      <c r="AG145" s="4"/>
+      <c r="AH145" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="AI145" s="16" t="s">
+      <c r="AI145" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="AJ145" s="16" t="s">
+      <c r="AJ145" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="AK145" s="16" t="s">
+      <c r="AK145" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="AL145" s="16" t="s">
+      <c r="AL145" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="AM145" s="16" t="s">
+      <c r="AM145" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="AN145" s="16" t="s">
+      <c r="AN145" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="AO145" s="16" t="s">
+      <c r="AO145" s="4" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="146" spans="33:41">
-      <c r="AG146" s="14" t="s">
+      <c r="AG146" t="s">
         <v>125</v>
       </c>
-      <c r="AH146" s="14">
+      <c r="AH146">
         <v>10.600953439555264</v>
       </c>
-      <c r="AI146" s="14">
+      <c r="AI146">
         <v>4.0881753464334878</v>
       </c>
-      <c r="AJ146" s="14">
+      <c r="AJ146">
         <v>2.5930769943132463</v>
       </c>
-      <c r="AK146" s="14">
+      <c r="AK146">
         <v>2.3524151066568539E-2</v>
       </c>
-      <c r="AL146" s="14">
+      <c r="AL146">
         <v>1.6935845448167139</v>
       </c>
-      <c r="AM146" s="14">
+      <c r="AM146">
         <v>19.508322334293815</v>
       </c>
-      <c r="AN146" s="14">
+      <c r="AN146">
         <v>1.6935845448167139</v>
       </c>
-      <c r="AO146" s="14">
+      <c r="AO146">
         <v>19.508322334293815</v>
       </c>
     </row>
-    <row r="147" spans="33:41" ht="15.75" thickBot="1">
-      <c r="AG147" s="15" t="s">
+    <row r="147" spans="33:41" ht="15" thickBot="1">
+      <c r="AG147" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="AH147" s="15">
+      <c r="AH147" s="3">
         <v>5.7666331750913999E-2</v>
       </c>
-      <c r="AI147" s="15">
+      <c r="AI147" s="3">
         <v>0.1350061928453978</v>
       </c>
-      <c r="AJ147" s="15">
+      <c r="AJ147" s="3">
         <v>0.42713841887942533</v>
       </c>
-      <c r="AK147" s="15">
+      <c r="AK147" s="3">
         <v>0.67684228954421743</v>
       </c>
-      <c r="AL147" s="15">
+      <c r="AL147" s="3">
         <v>-0.2364868933051667</v>
       </c>
-      <c r="AM147" s="15">
+      <c r="AM147" s="3">
         <v>0.35181955680699473</v>
       </c>
-      <c r="AN147" s="15">
+      <c r="AN147" s="3">
         <v>-0.2364868933051667</v>
       </c>
-      <c r="AO147" s="15">
+      <c r="AO147" s="3">
         <v>0.35181955680699473</v>
       </c>
     </row>
@@ -19913,209 +20083,207 @@
         <v>115</v>
       </c>
     </row>
-    <row r="151" spans="33:41" ht="15.75" thickBot="1"/>
+    <row r="151" spans="33:41" ht="15" thickBot="1"/>
     <row r="152" spans="33:41">
-      <c r="AG152" s="17" t="s">
+      <c r="AG152" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="AH152" s="17"/>
+      <c r="AH152" s="8"/>
     </row>
     <row r="153" spans="33:41">
-      <c r="AG153" s="14" t="s">
+      <c r="AG153" t="s">
         <v>117</v>
       </c>
-      <c r="AH153" s="14">
+      <c r="AH153">
         <v>0.70705776084779703</v>
       </c>
     </row>
     <row r="154" spans="33:41">
-      <c r="AG154" s="14" t="s">
+      <c r="AG154" t="s">
         <v>118</v>
       </c>
-      <c r="AH154" s="14">
+      <c r="AH154">
         <v>0.49993067717510059</v>
       </c>
     </row>
     <row r="155" spans="33:41">
-      <c r="AG155" s="14" t="s">
+      <c r="AG155" t="s">
         <v>119</v>
       </c>
-      <c r="AH155" s="14">
+      <c r="AH155">
         <v>0.45825823360635898</v>
       </c>
     </row>
     <row r="156" spans="33:41">
-      <c r="AG156" s="14" t="s">
+      <c r="AG156" t="s">
         <v>120</v>
       </c>
-      <c r="AH156" s="14">
+      <c r="AH156">
         <v>3.8929200651529965</v>
       </c>
     </row>
-    <row r="157" spans="33:41" ht="15.75" thickBot="1">
-      <c r="AG157" s="15" t="s">
+    <row r="157" spans="33:41" ht="15" thickBot="1">
+      <c r="AG157" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="AH157" s="15">
+      <c r="AH157" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="159" spans="33:41" ht="15.75" thickBot="1">
+    <row r="159" spans="33:41" ht="15" thickBot="1">
       <c r="AG159" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="160" spans="33:41">
-      <c r="AG160" s="16"/>
-      <c r="AH160" s="16" t="s">
+      <c r="AG160" s="4"/>
+      <c r="AH160" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="AI160" s="16" t="s">
+      <c r="AI160" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="AJ160" s="16" t="s">
+      <c r="AJ160" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="AK160" s="16" t="s">
+      <c r="AK160" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="AL160" s="20" t="s">
+      <c r="AL160" s="14" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="161" spans="33:41">
-      <c r="AG161" s="14" t="s">
+      <c r="AG161" t="s">
         <v>122</v>
       </c>
-      <c r="AH161" s="14">
+      <c r="AH161">
         <v>1</v>
       </c>
-      <c r="AI161" s="14">
+      <c r="AI161">
         <v>181.80749897578139</v>
       </c>
-      <c r="AJ161" s="14">
+      <c r="AJ161">
         <v>181.80749897578139</v>
       </c>
-      <c r="AK161" s="14">
+      <c r="AK161">
         <v>11.996672965683665</v>
       </c>
-      <c r="AL161" s="21">
+      <c r="AL161" s="6">
         <v>4.6857530529600564E-3</v>
       </c>
     </row>
     <row r="162" spans="33:41">
-      <c r="AG162" s="14" t="s">
+      <c r="AG162" t="s">
         <v>123</v>
       </c>
-      <c r="AH162" s="14">
+      <c r="AH162">
         <v>12</v>
       </c>
-      <c r="AI162" s="14">
+      <c r="AI162">
         <v>181.85791960404973</v>
       </c>
-      <c r="AJ162" s="14">
+      <c r="AJ162">
         <v>15.15482663367081</v>
       </c>
-      <c r="AK162" s="14"/>
-      <c r="AL162" s="14"/>
-    </row>
-    <row r="163" spans="33:41" ht="15.75" thickBot="1">
-      <c r="AG163" s="15" t="s">
+    </row>
+    <row r="163" spans="33:41" ht="15" thickBot="1">
+      <c r="AG163" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="AH163" s="15">
+      <c r="AH163" s="3">
         <v>13</v>
       </c>
-      <c r="AI163" s="15">
+      <c r="AI163" s="3">
         <v>363.66541857983111</v>
       </c>
-      <c r="AJ163" s="15"/>
-      <c r="AK163" s="15"/>
-      <c r="AL163" s="15"/>
-    </row>
-    <row r="164" spans="33:41" ht="15.75" thickBot="1"/>
+      <c r="AJ163" s="3"/>
+      <c r="AK163" s="3"/>
+      <c r="AL163" s="3"/>
+    </row>
+    <row r="164" spans="33:41" ht="15" thickBot="1"/>
     <row r="165" spans="33:41">
-      <c r="AG165" s="16"/>
-      <c r="AH165" s="16" t="s">
+      <c r="AG165" s="4"/>
+      <c r="AH165" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="AI165" s="16" t="s">
+      <c r="AI165" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="AJ165" s="16" t="s">
+      <c r="AJ165" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="AK165" s="16" t="s">
+      <c r="AK165" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="AL165" s="16" t="s">
+      <c r="AL165" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="AM165" s="16" t="s">
+      <c r="AM165" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="AN165" s="16" t="s">
+      <c r="AN165" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="AO165" s="16" t="s">
+      <c r="AO165" s="4" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="166" spans="33:41">
-      <c r="AG166" s="14" t="s">
+      <c r="AG166" t="s">
         <v>125</v>
       </c>
-      <c r="AH166" s="14">
+      <c r="AH166">
         <v>9.2047750648732709</v>
       </c>
-      <c r="AI166" s="14">
+      <c r="AI166">
         <v>2.9601302535842295</v>
       </c>
-      <c r="AJ166" s="14">
+      <c r="AJ166">
         <v>3.1095844697130492</v>
       </c>
-      <c r="AK166" s="14">
+      <c r="AK166">
         <v>9.0278090445263717E-3</v>
       </c>
-      <c r="AL166" s="14">
+      <c r="AL166">
         <v>2.7552052908778455</v>
       </c>
-      <c r="AM166" s="14">
+      <c r="AM166">
         <v>15.654344838868695</v>
       </c>
-      <c r="AN166" s="14">
+      <c r="AN166">
         <v>2.7552052908778455</v>
       </c>
-      <c r="AO166" s="14">
+      <c r="AO166">
         <v>15.654344838868695</v>
       </c>
     </row>
-    <row r="167" spans="33:41" ht="15.75" thickBot="1">
-      <c r="AG167" s="15" t="s">
+    <row r="167" spans="33:41" ht="15" thickBot="1">
+      <c r="AG167" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="AH167" s="15">
+      <c r="AH167" s="3">
         <v>0.33858320141151138</v>
       </c>
-      <c r="AI167" s="15">
+      <c r="AI167" s="3">
         <v>9.7754103480793705E-2</v>
       </c>
-      <c r="AJ167" s="15">
+      <c r="AJ167" s="3">
         <v>3.4636213658082875</v>
       </c>
-      <c r="AK167" s="15">
+      <c r="AK167" s="3">
         <v>4.6857530529600608E-3</v>
       </c>
-      <c r="AL167" s="15">
+      <c r="AL167" s="3">
         <v>0.12559530659494017</v>
       </c>
-      <c r="AM167" s="15">
+      <c r="AM167" s="3">
         <v>0.55157109622808265</v>
       </c>
-      <c r="AN167" s="15">
+      <c r="AN167" s="3">
         <v>0.12559530659494017</v>
       </c>
-      <c r="AO167" s="15">
+      <c r="AO167" s="3">
         <v>0.55157109622808265</v>
       </c>
     </row>
@@ -20132,19 +20300,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02490D31-8144-4D02-A37F-D0BDE3454DA1}">
-  <dimension ref="D2:AA34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="D2:Y34"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" customWidth="1"/>
-    <col min="11" max="11" width="12.85546875" customWidth="1"/>
-    <col min="12" max="12" width="16.5703125" customWidth="1"/>
-    <col min="13" max="13" width="18.140625" customWidth="1"/>
-    <col min="16" max="16" width="11.85546875" customWidth="1"/>
-    <col min="17" max="17" width="10.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" customWidth="1"/>
+    <col min="10" max="10" width="10.453125" customWidth="1"/>
+    <col min="11" max="11" width="12.81640625" customWidth="1"/>
+    <col min="12" max="12" width="16.54296875" customWidth="1"/>
+    <col min="13" max="13" width="18.1796875" customWidth="1"/>
+    <col min="16" max="16" width="11.81640625" customWidth="1"/>
+    <col min="17" max="17" width="10.453125" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" customWidth="1"/>
-    <col min="20" max="20" width="11.85546875" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" customWidth="1"/>
+    <col min="20" max="20" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="4:20">
@@ -20636,10 +20804,10 @@
         <v>0.62343700000000002</v>
       </c>
     </row>
-    <row r="17" spans="4:27">
+    <row r="17" spans="4:25">
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="4:27">
+    <row r="18" spans="4:25">
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
@@ -20656,26 +20824,14 @@
       <c r="R18" t="s">
         <v>174</v>
       </c>
-      <c r="V18" s="18"/>
-      <c r="W18" s="18"/>
-      <c r="X18" s="18"/>
-      <c r="Y18" s="18"/>
-      <c r="Z18" s="18"/>
-      <c r="AA18" s="18"/>
-    </row>
-    <row r="19" spans="4:27" ht="15.75" thickBot="1">
+    </row>
+    <row r="19" spans="4:25" ht="15" thickBot="1">
       <c r="H19" s="2"/>
       <c r="O19" t="s">
         <v>179</v>
       </c>
-      <c r="V19" s="18"/>
-      <c r="W19" s="18"/>
-      <c r="X19" s="18"/>
-      <c r="Y19" s="18"/>
-      <c r="Z19" s="18"/>
-      <c r="AA19" s="18"/>
-    </row>
-    <row r="20" spans="4:27">
+    </row>
+    <row r="20" spans="4:25">
       <c r="H20" s="2"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4" t="s">
@@ -20694,14 +20850,11 @@
       <c r="T20" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="V20" s="18"/>
-      <c r="W20" s="19"/>
-      <c r="X20" s="19"/>
-      <c r="Y20" s="19"/>
-      <c r="Z20" s="18"/>
-      <c r="AA20" s="18"/>
-    </row>
-    <row r="21" spans="4:27">
+      <c r="W20" s="9"/>
+      <c r="X20" s="9"/>
+      <c r="Y20" s="9"/>
+    </row>
+    <row r="21" spans="4:25">
       <c r="H21" s="2"/>
       <c r="J21" t="s">
         <v>99</v>
@@ -20721,14 +20874,8 @@
       <c r="T21">
         <v>0.5081012142857142</v>
       </c>
-      <c r="V21" s="18"/>
-      <c r="W21" s="14"/>
-      <c r="X21" s="14"/>
-      <c r="Y21" s="14"/>
-      <c r="Z21" s="18"/>
-      <c r="AA21" s="18"/>
-    </row>
-    <row r="22" spans="4:27">
+    </row>
+    <row r="22" spans="4:25">
       <c r="H22" s="2"/>
       <c r="J22" t="s">
         <v>100</v>
@@ -20748,14 +20895,8 @@
       <c r="T22">
         <v>1.4623475068181411E-2</v>
       </c>
-      <c r="V22" s="18"/>
-      <c r="W22" s="14"/>
-      <c r="X22" s="14"/>
-      <c r="Y22" s="14"/>
-      <c r="Z22" s="18"/>
-      <c r="AA22" s="18"/>
-    </row>
-    <row r="23" spans="4:27">
+    </row>
+    <row r="23" spans="4:25">
       <c r="H23" s="2"/>
       <c r="J23" t="s">
         <v>101</v>
@@ -20775,14 +20916,8 @@
       <c r="T23">
         <v>14</v>
       </c>
-      <c r="V23" s="18"/>
-      <c r="W23" s="14"/>
-      <c r="X23" s="14"/>
-      <c r="Y23" s="14"/>
-      <c r="Z23" s="18"/>
-      <c r="AA23" s="18"/>
-    </row>
-    <row r="24" spans="4:27">
+    </row>
+    <row r="24" spans="4:25">
       <c r="H24" s="2"/>
       <c r="J24" t="s">
         <v>103</v>
@@ -20799,14 +20934,8 @@
       <c r="S24">
         <v>0</v>
       </c>
-      <c r="V24" s="18"/>
-      <c r="W24" s="14"/>
-      <c r="X24" s="14"/>
-      <c r="Y24" s="14"/>
-      <c r="Z24" s="18"/>
-      <c r="AA24" s="18"/>
-    </row>
-    <row r="25" spans="4:27">
+    </row>
+    <row r="25" spans="4:25">
       <c r="H25" s="2"/>
       <c r="J25" t="s">
         <v>128</v>
@@ -20820,14 +20949,8 @@
       <c r="S25">
         <v>14</v>
       </c>
-      <c r="V25" s="18"/>
-      <c r="W25" s="14"/>
-      <c r="X25" s="14"/>
-      <c r="Y25" s="14"/>
-      <c r="Z25" s="18"/>
-      <c r="AA25" s="18"/>
-    </row>
-    <row r="26" spans="4:27">
+    </row>
+    <row r="26" spans="4:25">
       <c r="H26" s="2"/>
       <c r="J26" t="s">
         <v>161</v>
@@ -20841,14 +20964,8 @@
       <c r="S26">
         <v>1.3334667165923608</v>
       </c>
-      <c r="V26" s="18"/>
-      <c r="W26" s="14"/>
-      <c r="X26" s="14"/>
-      <c r="Y26" s="14"/>
-      <c r="Z26" s="18"/>
-      <c r="AA26" s="18"/>
-    </row>
-    <row r="27" spans="4:27" ht="15.75" thickBot="1">
+    </row>
+    <row r="27" spans="4:25" ht="15" thickBot="1">
       <c r="H27" s="2"/>
       <c r="J27" s="3" t="s">
         <v>162</v>
@@ -20863,42 +20980,24 @@
       <c r="S27">
         <v>0.10183490355630136</v>
       </c>
-      <c r="V27" s="18"/>
-      <c r="W27" s="14"/>
-      <c r="X27" s="14"/>
-      <c r="Y27" s="14"/>
-      <c r="Z27" s="18"/>
-      <c r="AA27" s="18"/>
-    </row>
-    <row r="28" spans="4:27">
+    </row>
+    <row r="28" spans="4:25">
       <c r="R28" t="s">
         <v>106</v>
       </c>
       <c r="S28">
         <v>1.7613101357748921</v>
       </c>
-      <c r="V28" s="18"/>
-      <c r="W28" s="14"/>
-      <c r="X28" s="14"/>
-      <c r="Y28" s="14"/>
-      <c r="Z28" s="18"/>
-      <c r="AA28" s="18"/>
-    </row>
-    <row r="29" spans="4:27">
+    </row>
+    <row r="29" spans="4:25">
       <c r="R29" t="s">
         <v>107</v>
       </c>
       <c r="S29">
         <v>0.20366980711260271</v>
       </c>
-      <c r="V29" s="18"/>
-      <c r="W29" s="14"/>
-      <c r="X29" s="14"/>
-      <c r="Y29" s="14"/>
-      <c r="Z29" s="18"/>
-      <c r="AA29" s="18"/>
-    </row>
-    <row r="30" spans="4:27" ht="15.75" thickBot="1">
+    </row>
+    <row r="30" spans="4:25" ht="15" thickBot="1">
       <c r="R30" s="3" t="s">
         <v>108</v>
       </c>
@@ -20906,38 +21005,8 @@
         <v>2.1447866879178044</v>
       </c>
       <c r="T30" s="3"/>
-      <c r="V30" s="18"/>
-      <c r="W30" s="14"/>
-      <c r="X30" s="14"/>
-      <c r="Y30" s="14"/>
-      <c r="Z30" s="18"/>
-      <c r="AA30" s="18"/>
-    </row>
-    <row r="31" spans="4:27">
-      <c r="V31" s="18"/>
-      <c r="W31" s="14"/>
-      <c r="X31" s="14"/>
-      <c r="Y31" s="14"/>
-      <c r="Z31" s="18"/>
-      <c r="AA31" s="18"/>
-    </row>
-    <row r="32" spans="4:27">
-      <c r="V32" s="18"/>
-      <c r="W32" s="18"/>
-      <c r="X32" s="18"/>
-      <c r="Y32" s="18"/>
-      <c r="Z32" s="18"/>
-      <c r="AA32" s="18"/>
-    </row>
-    <row r="33" spans="7:27">
-      <c r="V33" s="18"/>
-      <c r="W33" s="18"/>
-      <c r="X33" s="18"/>
-      <c r="Y33" s="18"/>
-      <c r="Z33" s="18"/>
-      <c r="AA33" s="18"/>
-    </row>
-    <row r="34" spans="7:27">
+    </row>
+    <row r="34" spans="7:9">
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
@@ -20956,15 +21025,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFC0AEBE-0304-40C9-AD55-B102AE5944DF}">
   <dimension ref="B1:T49"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
-    <col min="8" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" customWidth="1"/>
-    <col min="15" max="15" width="10.85546875" customWidth="1"/>
-    <col min="16" max="16" width="9.85546875" customWidth="1"/>
-    <col min="17" max="17" width="19.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" customWidth="1"/>
+    <col min="8" max="9" width="10.81640625" customWidth="1"/>
+    <col min="10" max="10" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" customWidth="1"/>
+    <col min="15" max="15" width="10.81640625" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" customWidth="1"/>
+    <col min="17" max="17" width="19.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:20">
@@ -21441,7 +21510,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="6:16" ht="15.75" thickBot="1">
+    <row r="20" spans="6:16" ht="15" thickBot="1">
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="6:16">
@@ -21572,7 +21641,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="6:16" ht="15.75" thickBot="1">
+    <row r="28" spans="6:16" ht="15" thickBot="1">
       <c r="F28" s="10"/>
       <c r="I28" s="3" t="s">
         <v>162</v>
@@ -21613,7 +21682,7 @@
         <v>1.6643182532567993E-2</v>
       </c>
     </row>
-    <row r="32" spans="6:16" ht="15.75" thickBot="1">
+    <row r="32" spans="6:16" ht="15" thickBot="1">
       <c r="N32" s="3" t="s">
         <v>108</v>
       </c>
@@ -21627,7 +21696,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="37" spans="2:4" ht="15.75" thickBot="1"/>
+    <row r="37" spans="2:4" ht="15" thickBot="1"/>
     <row r="38" spans="2:4">
       <c r="B38" s="4"/>
       <c r="C38" s="4" t="s">
@@ -21726,7 +21795,7 @@
         <v>4.3206917156444202E-2</v>
       </c>
     </row>
-    <row r="49" spans="2:4" ht="15.75" thickBot="1">
+    <row r="49" spans="2:4" ht="15" thickBot="1">
       <c r="B49" s="3" t="s">
         <v>108</v>
       </c>
@@ -21749,13 +21818,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D375B1A-F51E-4B8D-9DD1-817BE0164FEC}">
   <dimension ref="B1:AE31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" customWidth="1"/>
-    <col min="19" max="19" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" customWidth="1"/>
+    <col min="8" max="8" width="18.81640625" customWidth="1"/>
+    <col min="9" max="9" width="15.7265625" customWidth="1"/>
+    <col min="10" max="10" width="16.7265625" customWidth="1"/>
+    <col min="19" max="19" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:31">
@@ -22881,7 +22950,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="3:10" ht="15.75" thickBot="1">
+    <row r="19" spans="3:10" ht="15" thickBot="1">
       <c r="D19" t="s">
         <v>196</v>
       </c>
@@ -22896,187 +22965,329 @@
       </c>
     </row>
     <row r="20" spans="3:10">
-      <c r="C20" s="16"/>
-      <c r="D20" s="16" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16" t="s">
+      <c r="H20" s="4"/>
+      <c r="I20" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="J20" s="16" t="s">
+      <c r="J20" s="4" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="21" spans="3:10">
-      <c r="C21" s="14" t="s">
+      <c r="C21" t="s">
         <v>99</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21">
         <v>3.1866711818181814</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21">
         <v>4.7625588571428574</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="H21" t="s">
         <v>99</v>
       </c>
-      <c r="I21" s="14">
+      <c r="I21">
         <v>3.1866711818181814</v>
       </c>
-      <c r="J21" s="14">
+      <c r="J21">
         <v>4.7625588571428574</v>
       </c>
     </row>
     <row r="22" spans="3:10">
-      <c r="C22" s="14" t="s">
+      <c r="C22" t="s">
         <v>100</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22">
         <v>4.6360862014693662</v>
       </c>
-      <c r="E22" s="14">
+      <c r="E22">
         <v>5.7209807616301305</v>
       </c>
-      <c r="H22" s="14" t="s">
+      <c r="H22" t="s">
         <v>100</v>
       </c>
-      <c r="I22" s="14">
+      <c r="I22">
         <v>4.6360862014693662</v>
       </c>
-      <c r="J22" s="14">
+      <c r="J22">
         <v>5.7209807616301305</v>
       </c>
     </row>
     <row r="23" spans="3:10">
-      <c r="C23" s="14" t="s">
+      <c r="C23" t="s">
         <v>101</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23">
         <v>11</v>
       </c>
-      <c r="E23" s="14">
+      <c r="E23">
         <v>14</v>
       </c>
-      <c r="H23" s="14" t="s">
+      <c r="H23" t="s">
         <v>101</v>
       </c>
-      <c r="I23" s="14">
+      <c r="I23">
         <v>11</v>
       </c>
-      <c r="J23" s="14">
+      <c r="J23">
         <v>14</v>
       </c>
     </row>
     <row r="24" spans="3:10">
-      <c r="C24" s="14" t="s">
+      <c r="C24" t="s">
         <v>103</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24">
         <v>10</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24">
         <v>13</v>
       </c>
-      <c r="H24" s="14" t="s">
+      <c r="H24" t="s">
         <v>110</v>
       </c>
-      <c r="I24" s="14">
+      <c r="I24">
         <v>5.2492874746037117</v>
       </c>
-      <c r="J24" s="14"/>
     </row>
     <row r="25" spans="3:10">
-      <c r="C25" s="14" t="s">
+      <c r="C25" t="s">
         <v>128</v>
       </c>
-      <c r="D25" s="14">
+      <c r="D25">
         <v>0.81036563390721217</v>
       </c>
-      <c r="E25" s="14"/>
-      <c r="H25" s="14" t="s">
+      <c r="H25" t="s">
         <v>102</v>
       </c>
-      <c r="I25" s="14">
+      <c r="I25">
         <v>0</v>
       </c>
-      <c r="J25" s="14"/>
     </row>
     <row r="26" spans="3:10">
-      <c r="C26" s="14" t="s">
+      <c r="C26" t="s">
         <v>161</v>
       </c>
-      <c r="D26" s="14">
+      <c r="D26">
         <v>0.37531255241462402</v>
       </c>
-      <c r="E26" s="14"/>
-      <c r="H26" s="14" t="s">
+      <c r="H26" t="s">
         <v>103</v>
       </c>
-      <c r="I26" s="14">
+      <c r="I26">
         <v>23</v>
       </c>
-      <c r="J26" s="14"/>
-    </row>
-    <row r="27" spans="3:10" ht="15.75" thickBot="1">
-      <c r="C27" s="15" t="s">
+    </row>
+    <row r="27" spans="3:10" ht="15" thickBot="1">
+      <c r="C27" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="3">
         <v>0.34635936731356898</v>
       </c>
-      <c r="E27" s="15"/>
-      <c r="H27" s="14" t="s">
+      <c r="E27" s="3"/>
+      <c r="H27" t="s">
         <v>104</v>
       </c>
-      <c r="I27" s="14">
+      <c r="I27">
         <v>-1.7071254481459661</v>
       </c>
-      <c r="J27" s="14"/>
     </row>
     <row r="28" spans="3:10">
-      <c r="H28" s="14" t="s">
+      <c r="H28" t="s">
         <v>105</v>
       </c>
-      <c r="I28" s="14">
+      <c r="I28">
         <v>5.0632689909300602E-2</v>
       </c>
-      <c r="J28" s="14"/>
     </row>
     <row r="29" spans="3:10">
-      <c r="H29" s="14" t="s">
+      <c r="H29" t="s">
         <v>106</v>
       </c>
-      <c r="I29" s="14">
+      <c r="I29">
         <v>1.7138715277470482</v>
       </c>
-      <c r="J29" s="14"/>
     </row>
     <row r="30" spans="3:10">
-      <c r="H30" s="14" t="s">
+      <c r="H30" t="s">
         <v>107</v>
       </c>
-      <c r="I30" s="14">
+      <c r="I30">
         <v>0.101265379818601</v>
       </c>
-      <c r="J30" s="14"/>
-    </row>
-    <row r="31" spans="3:10" ht="15.75" thickBot="1">
-      <c r="H31" s="15" t="s">
+    </row>
+    <row r="31" spans="3:10" ht="15" thickBot="1">
+      <c r="H31" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="I31" s="15">
+      <c r="I31" s="3">
         <v>2.0686576104190491</v>
       </c>
-      <c r="J31" s="15"/>
+      <c r="J31" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2EABC84-23BA-464A-9765-728455CFA12E}">
+  <dimension ref="B3:G17"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="14.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="23.6328125" customWidth="1"/>
+    <col min="5" max="5" width="24.36328125" customWidth="1"/>
+    <col min="6" max="6" width="23.08984375" customWidth="1"/>
+    <col min="7" max="7" width="27" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" ht="29">
+      <c r="B3" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="43.5">
+      <c r="B4" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="409.5">
+      <c r="B5" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="58">
+      <c r="B6" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="29">
+      <c r="B7" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+    </row>
+    <row r="8" spans="2:7">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+    </row>
+    <row r="9" spans="2:7">
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+    </row>
+    <row r="13" spans="2:7">
+      <c r="D13" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="D14" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7">
+      <c r="D15" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7">
+      <c r="D16" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="17" spans="4:4">
+      <c r="D17" t="s">
+        <v>234</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>

</xml_diff>